<commit_message>
Valley Triad: populate card roster with real SDV objects (52 cards)
Filled cards.xlsx from the wiki category data: 24 Common (crops with correct
seasons, forageables, animals, quartz), 15 Uncommon (villagers), 8 Rare
(monsters, minerals, Ancient Fruit, Sturgeon, Sweet Gem Berry), 5 Legendary
(Wizard, Junimo King, Mr. Qi, Crimsonfish, Prismatic Shard). Seasons from the
Crops/Foraging pages; sprite refs use legacy object IDs / Villager|Animal|
Monster|Special tags. All stat lines validated within tier edge budgets.
</commit_message>
<xml_diff>
--- a/ValleyTriad/cards.xlsx
+++ b/ValleyTriad/cards.xlsx
@@ -518,7 +518,7 @@
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -614,7 +614,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>monstros, artesanais, NPCs especiais</t>
+          <t>monstros, minerais, peixes/goods especiais</t>
         </is>
       </c>
     </row>
@@ -635,14 +635,14 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Mago, Rei Junimo, Peixe Lendário, Sr. Qi</t>
+          <t>Mago, Rei Junimo, Sr. Qi, peixe lendário, Frag. Prismático</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Cada carta tem 4 bordas (N/L/S/O), valores de 1 a 10 (10 = 'A'). A soma das 4 deve cair na faixa do tier.</t>
+          <t>Cada carta tem 4 bordas (N/L/S/O), 1 a 10 (10 = 'A'). A soma das 4 deve cair na faixa do tier.</t>
         </is>
       </c>
     </row>
@@ -657,37 +657,37 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O56"/>
+  <dimension ref="A1:O62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
     <col width="5" customWidth="1" min="8" max="8"/>
     <col width="5" customWidth="1" min="9" max="9"/>
     <col width="5" customWidth="1" min="10" max="10"/>
     <col width="5" customWidth="1" min="11" max="11"/>
     <col width="7" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
-    <col width="30" customWidth="1" min="15" max="15"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="15" customWidth="1" min="14" max="14"/>
+    <col width="26" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Valley Triad — Acervo de cartas (v1, ~50)</t>
+          <t>Valley Triad — Acervo de cartas (v1)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>Preencha N/L/S/O (1–10). 'Soma' e 'Orçamento?' são automáticos. 'Sprite' = de onde puxar a imagem em runtime (ex.: (O)24, Villager:Abigail).</t>
+          <t>Objetos reais do SDV (wiki). Sprite = de onde puxar a imagem em runtime: (O)&lt;id&gt; objeto · Villager:&lt;Nome&gt; · Animal:&lt;Tipo&gt; · Monster:&lt;Tipo&gt; · Special:&lt;Nome&gt;. 'Soma' e 'Orçamento?' são automáticos.</t>
         </is>
       </c>
     </row>
@@ -900,12 +900,12 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Blueberry</t>
+          <t>Potato</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Mirtilo</t>
+          <t>Batata</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -920,25 +920,25 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Verão</t>
+          <t>Primavera</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>(O)258</t>
+          <t>(O)192</t>
         </is>
       </c>
       <c r="H7" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J7" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="K7" s="4" t="n">
         <v>2</v>
-      </c>
-      <c r="I7" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="J7" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="K7" s="4" t="n">
-        <v>4</v>
       </c>
       <c r="L7" s="4">
         <f>IF(COUNT(H7:K7)=4,SUM(H7:K7),"")</f>
@@ -961,12 +961,12 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Pumpkin</t>
+          <t>Green Bean</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Abóbora</t>
+          <t>Vagem</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -981,22 +981,22 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Outono</t>
+          <t>Primavera</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>(O)276</t>
+          <t>(O)188</t>
         </is>
       </c>
       <c r="H8" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="J8" s="4" t="n">
         <v>3</v>
-      </c>
-      <c r="J8" s="4" t="n">
-        <v>4</v>
       </c>
       <c r="K8" s="4" t="n">
         <v>2</v>
@@ -1011,14 +1011,10 @@
       </c>
       <c r="N8" s="5" t="inlineStr">
         <is>
-          <t>Pacote inicial</t>
-        </is>
-      </c>
-      <c r="O8" s="5" t="inlineStr">
-        <is>
-          <t>boa em casa de Outono</t>
-        </is>
-      </c>
+          <t>Ganhar de NPC</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
@@ -1026,17 +1022,17 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Salmonberry</t>
+          <t>Blueberry</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Amora-salmão</t>
+          <t>Mirtilo</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Forrageável</t>
+          <t>Crop</t>
         </is>
       </c>
       <c r="E9" s="10" t="inlineStr">
@@ -1046,25 +1042,25 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Primavera</t>
+          <t>Verão</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>(O)296</t>
+          <t>(O)258</t>
         </is>
       </c>
       <c r="H9" s="4" t="n">
         <v>2</v>
       </c>
       <c r="I9" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="J9" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="J9" s="4" t="n">
-        <v>2</v>
-      </c>
       <c r="K9" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L9" s="4">
         <f>IF(COUNT(H9:K9)=4,SUM(H9:K9),"")</f>
@@ -1076,7 +1072,7 @@
       </c>
       <c r="N9" s="5" t="inlineStr">
         <is>
-          <t>Ganhar de NPC</t>
+          <t>Pacote inicial</t>
         </is>
       </c>
       <c r="O9" s="5" t="inlineStr"/>
@@ -1087,17 +1083,17 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Common Mushroom</t>
+          <t>Hot Pepper</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Cogumelo Comum</t>
+          <t>Pimenta</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Forrageável</t>
+          <t>Crop</t>
         </is>
       </c>
       <c r="E10" s="10" t="inlineStr">
@@ -1107,25 +1103,25 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Outono</t>
+          <t>Verão</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>(O)404</t>
+          <t>(O)260</t>
         </is>
       </c>
       <c r="H10" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I10" s="4" t="n">
         <v>2</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L10" s="4">
         <f>IF(COUNT(H10:K10)=4,SUM(H10:K10),"")</f>
@@ -1148,17 +1144,17 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Chicken</t>
+          <t>Melon</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Galinha</t>
+          <t>Melão</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Animal</t>
+          <t>Crop</t>
         </is>
       </c>
       <c r="E11" s="10" t="inlineStr">
@@ -1168,22 +1164,22 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Nenhum</t>
+          <t>Verão</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Animal:Chicken</t>
+          <t>(O)254</t>
         </is>
       </c>
       <c r="H11" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I11" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J11" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K11" s="4" t="n">
         <v>3</v>
@@ -1198,7 +1194,7 @@
       </c>
       <c r="N11" s="5" t="inlineStr">
         <is>
-          <t>Pacote inicial</t>
+          <t>Ganhar de NPC</t>
         </is>
       </c>
       <c r="O11" s="5" t="inlineStr"/>
@@ -1209,17 +1205,17 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Cow</t>
+          <t>Tomato</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Vaca</t>
+          <t>Tomate</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Animal</t>
+          <t>Crop</t>
         </is>
       </c>
       <c r="E12" s="10" t="inlineStr">
@@ -1229,25 +1225,25 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Nenhum</t>
+          <t>Verão</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Animal:Cow</t>
+          <t>(O)256</t>
         </is>
       </c>
       <c r="H12" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J12" s="4" t="n">
         <v>3</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L12" s="4">
         <f>IF(COUNT(H12:K12)=4,SUM(H12:K12),"")</f>
@@ -1259,7 +1255,7 @@
       </c>
       <c r="N12" s="5" t="inlineStr">
         <is>
-          <t>Ganhar de NPC</t>
+          <t>Pacote inicial</t>
         </is>
       </c>
       <c r="O12" s="5" t="inlineStr"/>
@@ -1270,17 +1266,17 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Green Slime</t>
+          <t>Pumpkin</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Slime Verde</t>
+          <t>Abóbora</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Monstro</t>
+          <t>Crop</t>
         </is>
       </c>
       <c r="E13" s="10" t="inlineStr">
@@ -1290,25 +1286,25 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Nenhum</t>
+          <t>Outono</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Monster:GreenSlime</t>
+          <t>(O)276</t>
         </is>
       </c>
       <c r="H13" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="I13" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J13" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="K13" s="4" t="n">
         <v>2</v>
-      </c>
-      <c r="I13" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="J13" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="K13" s="4" t="n">
-        <v>1</v>
       </c>
       <c r="L13" s="4">
         <f>IF(COUNT(H13:K13)=4,SUM(H13:K13),"")</f>
@@ -1323,7 +1319,11 @@
           <t>Ganhar de NPC</t>
         </is>
       </c>
-      <c r="O13" s="5" t="inlineStr"/>
+      <c r="O13" s="5" t="inlineStr">
+        <is>
+          <t>forte em casa de Outono</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
@@ -1331,45 +1331,45 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Abigail</t>
+          <t>Cranberries</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Abigail</t>
+          <t>Oxicoco</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Aldeão</t>
-        </is>
-      </c>
-      <c r="E14" s="11" t="inlineStr">
-        <is>
-          <t>Incomum</t>
+          <t>Crop</t>
+        </is>
+      </c>
+      <c r="E14" s="10" t="inlineStr">
+        <is>
+          <t>Comum</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Nenhum</t>
+          <t>Outono</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>Villager:Abigail</t>
+          <t>(O)282</t>
         </is>
       </c>
       <c r="H14" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J14" s="4" t="n">
         <v>4</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L14" s="4">
         <f>IF(COUNT(H14:K14)=4,SUM(H14:K14),"")</f>
@@ -1384,11 +1384,7 @@
           <t>Ganhar de NPC</t>
         </is>
       </c>
-      <c r="O14" s="5" t="inlineStr">
-        <is>
-          <t>mentora / evento inicial</t>
-        </is>
-      </c>
+      <c r="O14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
@@ -1396,45 +1392,45 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Sebastian</t>
+          <t>Eggplant</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Sebastian</t>
+          <t>Berinjela</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Aldeão</t>
-        </is>
-      </c>
-      <c r="E15" s="11" t="inlineStr">
-        <is>
-          <t>Incomum</t>
+          <t>Crop</t>
+        </is>
+      </c>
+      <c r="E15" s="10" t="inlineStr">
+        <is>
+          <t>Comum</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Nenhum</t>
+          <t>Outono</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>Villager:Sebastian</t>
+          <t>(O)272</t>
         </is>
       </c>
       <c r="H15" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I15" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J15" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K15" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L15" s="4">
         <f>IF(COUNT(H15:K15)=4,SUM(H15:K15),"")</f>
@@ -1457,45 +1453,45 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Gus</t>
+          <t>Yam</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Gus</t>
+          <t>Inhame</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Aldeão</t>
-        </is>
-      </c>
-      <c r="E16" s="11" t="inlineStr">
-        <is>
-          <t>Incomum</t>
+          <t>Crop</t>
+        </is>
+      </c>
+      <c r="E16" s="10" t="inlineStr">
+        <is>
+          <t>Comum</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>Nenhum</t>
+          <t>Outono</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Villager:Gus</t>
+          <t>(O)280</t>
         </is>
       </c>
       <c r="H16" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I16" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J16" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K16" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L16" s="4">
         <f>IF(COUNT(H16:K16)=4,SUM(H16:K16),"")</f>
@@ -1507,14 +1503,10 @@
       </c>
       <c r="N16" s="5" t="inlineStr">
         <is>
-          <t>Ganhar de NPC</t>
-        </is>
-      </c>
-      <c r="O16" s="5" t="inlineStr">
-        <is>
-          <t>dono do Saloon</t>
-        </is>
-      </c>
+          <t>Pacote inicial</t>
+        </is>
+      </c>
+      <c r="O16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
@@ -1522,45 +1514,45 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Skeleton</t>
+          <t>Wild Horseradish</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Esqueleto</t>
+          <t>Raiz-forte silvestre</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Monstro</t>
-        </is>
-      </c>
-      <c r="E17" s="12" t="inlineStr">
-        <is>
-          <t>Raro</t>
+          <t>Forrageável</t>
+        </is>
+      </c>
+      <c r="E17" s="10" t="inlineStr">
+        <is>
+          <t>Comum</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Nenhum</t>
+          <t>Primavera</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>Monster:Skeleton</t>
+          <t>(O)16</t>
         </is>
       </c>
       <c r="H17" s="4" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I17" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J17" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K17" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="L17" s="4">
         <f>IF(COUNT(H17:K17)=4,SUM(H17:K17),"")</f>
@@ -1583,45 +1575,45 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Prismatic Shard</t>
+          <t>Salmonberry</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Fragmento Prismático</t>
+          <t>Amora-salmão</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Mineral</t>
-        </is>
-      </c>
-      <c r="E18" s="12" t="inlineStr">
-        <is>
-          <t>Raro</t>
+          <t>Forrageável</t>
+        </is>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
+        <is>
+          <t>Comum</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Nenhum</t>
+          <t>Primavera</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>(O)74</t>
+          <t>(O)296</t>
         </is>
       </c>
       <c r="H18" s="4" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="I18" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="J18" s="4" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="K18" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L18" s="4">
         <f>IF(COUNT(H18:K18)=4,SUM(H18:K18),"")</f>
@@ -1644,45 +1636,45 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Wizard</t>
+          <t>Spice Berry</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Mago</t>
+          <t>Baga Picante</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Especial</t>
-        </is>
-      </c>
-      <c r="E19" s="13" t="inlineStr">
-        <is>
-          <t>Lendário</t>
+          <t>Forrageável</t>
+        </is>
+      </c>
+      <c r="E19" s="10" t="inlineStr">
+        <is>
+          <t>Comum</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>Nenhum</t>
+          <t>Verão</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Villager:Wizard</t>
+          <t>(O)396</t>
         </is>
       </c>
       <c r="H19" s="4" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="I19" s="4" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="J19" s="4" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="K19" s="4" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="L19" s="4">
         <f>IF(COUNT(H19:K19)=4,SUM(H19:K19),"")</f>
@@ -1694,14 +1686,10 @@
       </c>
       <c r="N19" s="5" t="inlineStr">
         <is>
-          <t>Campeão</t>
-        </is>
-      </c>
-      <c r="O19" s="5" t="inlineStr">
-        <is>
-          <t>boss</t>
-        </is>
-      </c>
+          <t>Ganhar de NPC</t>
+        </is>
+      </c>
+      <c r="O19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
@@ -1709,45 +1697,45 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Junimo King</t>
+          <t>Common Mushroom</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Rei Junimo</t>
+          <t>Cogumelo Comum</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Especial</t>
-        </is>
-      </c>
-      <c r="E20" s="13" t="inlineStr">
-        <is>
-          <t>Lendário</t>
+          <t>Forrageável</t>
+        </is>
+      </c>
+      <c r="E20" s="10" t="inlineStr">
+        <is>
+          <t>Comum</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>Nenhum</t>
+          <t>Outono</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>Special:JunimoKing</t>
+          <t>(O)404</t>
         </is>
       </c>
       <c r="H20" s="4" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="I20" s="4" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="L20" s="4">
         <f>IF(COUNT(H20:K20)=4,SUM(H20:K20),"")</f>
@@ -1759,14 +1747,10 @@
       </c>
       <c r="N20" s="5" t="inlineStr">
         <is>
-          <t>Campeão</t>
-        </is>
-      </c>
-      <c r="O20" s="5" t="inlineStr">
-        <is>
-          <t>boss</t>
-        </is>
-      </c>
+          <t>Ganhar de NPC</t>
+        </is>
+      </c>
+      <c r="O20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
@@ -1774,45 +1758,45 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Mr. Qi</t>
+          <t>Blackberry</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Sr. Qi</t>
+          <t>Amora-preta</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Especial</t>
-        </is>
-      </c>
-      <c r="E21" s="13" t="inlineStr">
-        <is>
-          <t>Lendário</t>
+          <t>Forrageável</t>
+        </is>
+      </c>
+      <c r="E21" s="10" t="inlineStr">
+        <is>
+          <t>Comum</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>Nenhum</t>
+          <t>Outono</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>Villager:Qi</t>
+          <t>(O)410</t>
         </is>
       </c>
       <c r="H21" s="4" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="I21" s="4" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J21" s="4" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="K21" s="4" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="L21" s="4">
         <f>IF(COUNT(H21:K21)=4,SUM(H21:K21),"")</f>
@@ -1824,27 +1808,57 @@
       </c>
       <c r="N21" s="5" t="inlineStr">
         <is>
-          <t>Campeão</t>
-        </is>
-      </c>
-      <c r="O21" s="5" t="inlineStr">
-        <is>
-          <t>boss</t>
-        </is>
-      </c>
+          <t>Ganhar de NPC</t>
+        </is>
+      </c>
+      <c r="O21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="inlineStr"/>
-      <c r="B22" s="5" t="inlineStr"/>
-      <c r="C22" s="5" t="inlineStr"/>
-      <c r="D22" s="5" t="inlineStr"/>
-      <c r="E22" s="4" t="inlineStr"/>
-      <c r="F22" s="4" t="inlineStr"/>
-      <c r="G22" s="5" t="inlineStr"/>
-      <c r="H22" s="4" t="inlineStr"/>
-      <c r="I22" s="4" t="inlineStr"/>
-      <c r="J22" s="4" t="inlineStr"/>
-      <c r="K22" s="4" t="inlineStr"/>
+      <c r="A22" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Winter Root</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Raiz de Inverno</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Forrageável</t>
+        </is>
+      </c>
+      <c r="E22" s="10" t="inlineStr">
+        <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>Inverno</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>(O)412</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I22" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J22" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K22" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="L22" s="4">
         <f>IF(COUNT(H22:K22)=4,SUM(H22:K22),"")</f>
         <v/>
@@ -1853,21 +1867,59 @@
         <f>IF(OR(E22="",L22=""),"",IF(AND(L22&gt;=VLOOKUP(E22,Tiers!$A$4:$C$7,2,0),L22&lt;=VLOOKUP(E22,Tiers!$A$4:$C$7,3,0)),"OK","Fora"))</f>
         <v/>
       </c>
-      <c r="N22" s="5" t="n"/>
-      <c r="O22" s="5" t="n"/>
+      <c r="N22" s="5" t="inlineStr">
+        <is>
+          <t>Ganhar de NPC</t>
+        </is>
+      </c>
+      <c r="O22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="inlineStr"/>
-      <c r="B23" s="5" t="inlineStr"/>
-      <c r="C23" s="5" t="inlineStr"/>
-      <c r="D23" s="5" t="inlineStr"/>
-      <c r="E23" s="4" t="inlineStr"/>
-      <c r="F23" s="4" t="inlineStr"/>
-      <c r="G23" s="5" t="inlineStr"/>
-      <c r="H23" s="4" t="inlineStr"/>
-      <c r="I23" s="4" t="inlineStr"/>
-      <c r="J23" s="4" t="inlineStr"/>
-      <c r="K23" s="4" t="inlineStr"/>
+      <c r="A23" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Snow Yam</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Inhame da Neve</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Forrageável</t>
+        </is>
+      </c>
+      <c r="E23" s="10" t="inlineStr">
+        <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>Inverno</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>(O)416</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I23" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J23" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="K23" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="L23" s="4">
         <f>IF(COUNT(H23:K23)=4,SUM(H23:K23),"")</f>
         <v/>
@@ -1876,21 +1928,59 @@
         <f>IF(OR(E23="",L23=""),"",IF(AND(L23&gt;=VLOOKUP(E23,Tiers!$A$4:$C$7,2,0),L23&lt;=VLOOKUP(E23,Tiers!$A$4:$C$7,3,0)),"OK","Fora"))</f>
         <v/>
       </c>
-      <c r="N23" s="5" t="n"/>
-      <c r="O23" s="5" t="n"/>
+      <c r="N23" s="5" t="inlineStr">
+        <is>
+          <t>Ganhar de NPC</t>
+        </is>
+      </c>
+      <c r="O23" s="5" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="inlineStr"/>
-      <c r="B24" s="5" t="inlineStr"/>
-      <c r="C24" s="5" t="inlineStr"/>
-      <c r="D24" s="5" t="inlineStr"/>
-      <c r="E24" s="4" t="inlineStr"/>
-      <c r="F24" s="4" t="inlineStr"/>
-      <c r="G24" s="5" t="inlineStr"/>
-      <c r="H24" s="4" t="inlineStr"/>
-      <c r="I24" s="4" t="inlineStr"/>
-      <c r="J24" s="4" t="inlineStr"/>
-      <c r="K24" s="4" t="inlineStr"/>
+      <c r="A24" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Chicken</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Galinha</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Animal</t>
+        </is>
+      </c>
+      <c r="E24" s="10" t="inlineStr">
+        <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>Nenhum</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>Animal:Chicken</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I24" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J24" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="K24" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="L24" s="4">
         <f>IF(COUNT(H24:K24)=4,SUM(H24:K24),"")</f>
         <v/>
@@ -1899,21 +1989,59 @@
         <f>IF(OR(E24="",L24=""),"",IF(AND(L24&gt;=VLOOKUP(E24,Tiers!$A$4:$C$7,2,0),L24&lt;=VLOOKUP(E24,Tiers!$A$4:$C$7,3,0)),"OK","Fora"))</f>
         <v/>
       </c>
-      <c r="N24" s="5" t="n"/>
-      <c r="O24" s="5" t="n"/>
+      <c r="N24" s="5" t="inlineStr">
+        <is>
+          <t>Pacote inicial</t>
+        </is>
+      </c>
+      <c r="O24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="4" t="inlineStr"/>
-      <c r="B25" s="5" t="inlineStr"/>
-      <c r="C25" s="5" t="inlineStr"/>
-      <c r="D25" s="5" t="inlineStr"/>
-      <c r="E25" s="4" t="inlineStr"/>
-      <c r="F25" s="4" t="inlineStr"/>
-      <c r="G25" s="5" t="inlineStr"/>
-      <c r="H25" s="4" t="inlineStr"/>
-      <c r="I25" s="4" t="inlineStr"/>
-      <c r="J25" s="4" t="inlineStr"/>
-      <c r="K25" s="4" t="inlineStr"/>
+      <c r="A25" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Cow</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Vaca</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Animal</t>
+        </is>
+      </c>
+      <c r="E25" s="10" t="inlineStr">
+        <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>Nenhum</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>Animal:Cow</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="I25" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J25" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="K25" s="4" t="n">
+        <v>4</v>
+      </c>
       <c r="L25" s="4">
         <f>IF(COUNT(H25:K25)=4,SUM(H25:K25),"")</f>
         <v/>
@@ -1922,21 +2050,59 @@
         <f>IF(OR(E25="",L25=""),"",IF(AND(L25&gt;=VLOOKUP(E25,Tiers!$A$4:$C$7,2,0),L25&lt;=VLOOKUP(E25,Tiers!$A$4:$C$7,3,0)),"OK","Fora"))</f>
         <v/>
       </c>
-      <c r="N25" s="5" t="n"/>
-      <c r="O25" s="5" t="n"/>
+      <c r="N25" s="5" t="inlineStr">
+        <is>
+          <t>Ganhar de NPC</t>
+        </is>
+      </c>
+      <c r="O25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="inlineStr"/>
-      <c r="B26" s="5" t="inlineStr"/>
-      <c r="C26" s="5" t="inlineStr"/>
-      <c r="D26" s="5" t="inlineStr"/>
-      <c r="E26" s="4" t="inlineStr"/>
-      <c r="F26" s="4" t="inlineStr"/>
-      <c r="G26" s="5" t="inlineStr"/>
-      <c r="H26" s="4" t="inlineStr"/>
-      <c r="I26" s="4" t="inlineStr"/>
-      <c r="J26" s="4" t="inlineStr"/>
-      <c r="K26" s="4" t="inlineStr"/>
+      <c r="A26" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Duck</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Pato</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Animal</t>
+        </is>
+      </c>
+      <c r="E26" s="10" t="inlineStr">
+        <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>Nenhum</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>Animal:Duck</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I26" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J26" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="K26" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="L26" s="4">
         <f>IF(COUNT(H26:K26)=4,SUM(H26:K26),"")</f>
         <v/>
@@ -1945,21 +2111,59 @@
         <f>IF(OR(E26="",L26=""),"",IF(AND(L26&gt;=VLOOKUP(E26,Tiers!$A$4:$C$7,2,0),L26&lt;=VLOOKUP(E26,Tiers!$A$4:$C$7,3,0)),"OK","Fora"))</f>
         <v/>
       </c>
-      <c r="N26" s="5" t="n"/>
-      <c r="O26" s="5" t="n"/>
+      <c r="N26" s="5" t="inlineStr">
+        <is>
+          <t>Ganhar de NPC</t>
+        </is>
+      </c>
+      <c r="O26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="4" t="inlineStr"/>
-      <c r="B27" s="5" t="inlineStr"/>
-      <c r="C27" s="5" t="inlineStr"/>
-      <c r="D27" s="5" t="inlineStr"/>
-      <c r="E27" s="4" t="inlineStr"/>
-      <c r="F27" s="4" t="inlineStr"/>
-      <c r="G27" s="5" t="inlineStr"/>
-      <c r="H27" s="4" t="inlineStr"/>
-      <c r="I27" s="4" t="inlineStr"/>
-      <c r="J27" s="4" t="inlineStr"/>
-      <c r="K27" s="4" t="inlineStr"/>
+      <c r="A27" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Rabbit</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Coelho</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>Animal</t>
+        </is>
+      </c>
+      <c r="E27" s="10" t="inlineStr">
+        <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>Nenhum</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>Animal:Rabbit</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I27" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="J27" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="K27" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="L27" s="4">
         <f>IF(COUNT(H27:K27)=4,SUM(H27:K27),"")</f>
         <v/>
@@ -1968,21 +2172,59 @@
         <f>IF(OR(E27="",L27=""),"",IF(AND(L27&gt;=VLOOKUP(E27,Tiers!$A$4:$C$7,2,0),L27&lt;=VLOOKUP(E27,Tiers!$A$4:$C$7,3,0)),"OK","Fora"))</f>
         <v/>
       </c>
-      <c r="N27" s="5" t="n"/>
-      <c r="O27" s="5" t="n"/>
+      <c r="N27" s="5" t="inlineStr">
+        <is>
+          <t>Ganhar de NPC</t>
+        </is>
+      </c>
+      <c r="O27" s="5" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="4" t="inlineStr"/>
-      <c r="B28" s="5" t="inlineStr"/>
-      <c r="C28" s="5" t="inlineStr"/>
-      <c r="D28" s="5" t="inlineStr"/>
-      <c r="E28" s="4" t="inlineStr"/>
-      <c r="F28" s="4" t="inlineStr"/>
-      <c r="G28" s="5" t="inlineStr"/>
-      <c r="H28" s="4" t="inlineStr"/>
-      <c r="I28" s="4" t="inlineStr"/>
-      <c r="J28" s="4" t="inlineStr"/>
-      <c r="K28" s="4" t="inlineStr"/>
+      <c r="A28" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Quartz</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Quartzo</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Mineral</t>
+        </is>
+      </c>
+      <c r="E28" s="10" t="inlineStr">
+        <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>Nenhum</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>(O)80</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I28" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J28" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K28" s="4" t="n">
+        <v>4</v>
+      </c>
       <c r="L28" s="4">
         <f>IF(COUNT(H28:K28)=4,SUM(H28:K28),"")</f>
         <v/>
@@ -1991,21 +2233,59 @@
         <f>IF(OR(E28="",L28=""),"",IF(AND(L28&gt;=VLOOKUP(E28,Tiers!$A$4:$C$7,2,0),L28&lt;=VLOOKUP(E28,Tiers!$A$4:$C$7,3,0)),"OK","Fora"))</f>
         <v/>
       </c>
-      <c r="N28" s="5" t="n"/>
-      <c r="O28" s="5" t="n"/>
+      <c r="N28" s="5" t="inlineStr">
+        <is>
+          <t>Ganhar de NPC</t>
+        </is>
+      </c>
+      <c r="O28" s="5" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="inlineStr"/>
-      <c r="B29" s="5" t="inlineStr"/>
-      <c r="C29" s="5" t="inlineStr"/>
-      <c r="D29" s="5" t="inlineStr"/>
-      <c r="E29" s="4" t="inlineStr"/>
-      <c r="F29" s="4" t="inlineStr"/>
-      <c r="G29" s="5" t="inlineStr"/>
-      <c r="H29" s="4" t="inlineStr"/>
-      <c r="I29" s="4" t="inlineStr"/>
-      <c r="J29" s="4" t="inlineStr"/>
-      <c r="K29" s="4" t="inlineStr"/>
+      <c r="A29" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Abigail</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>Abigail</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>Aldeão</t>
+        </is>
+      </c>
+      <c r="E29" s="11" t="inlineStr">
+        <is>
+          <t>Incomum</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>Nenhum</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>Villager:Abigail</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="I29" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J29" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="K29" s="4" t="n">
+        <v>5</v>
+      </c>
       <c r="L29" s="4">
         <f>IF(COUNT(H29:K29)=4,SUM(H29:K29),"")</f>
         <v/>
@@ -2014,21 +2294,63 @@
         <f>IF(OR(E29="",L29=""),"",IF(AND(L29&gt;=VLOOKUP(E29,Tiers!$A$4:$C$7,2,0),L29&lt;=VLOOKUP(E29,Tiers!$A$4:$C$7,3,0)),"OK","Fora"))</f>
         <v/>
       </c>
-      <c r="N29" s="5" t="n"/>
-      <c r="O29" s="5" t="n"/>
+      <c r="N29" s="5" t="inlineStr">
+        <is>
+          <t>Ganhar de NPC</t>
+        </is>
+      </c>
+      <c r="O29" s="5" t="inlineStr">
+        <is>
+          <t>mentora / evento inicial</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="inlineStr"/>
-      <c r="B30" s="5" t="inlineStr"/>
-      <c r="C30" s="5" t="inlineStr"/>
-      <c r="D30" s="5" t="inlineStr"/>
-      <c r="E30" s="4" t="inlineStr"/>
-      <c r="F30" s="4" t="inlineStr"/>
-      <c r="G30" s="5" t="inlineStr"/>
-      <c r="H30" s="4" t="inlineStr"/>
-      <c r="I30" s="4" t="inlineStr"/>
-      <c r="J30" s="4" t="inlineStr"/>
-      <c r="K30" s="4" t="inlineStr"/>
+      <c r="A30" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Sebastian</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Sebastian</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Aldeão</t>
+        </is>
+      </c>
+      <c r="E30" s="11" t="inlineStr">
+        <is>
+          <t>Incomum</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>Nenhum</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>Villager:Sebastian</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I30" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="J30" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="K30" s="4" t="n">
+        <v>4</v>
+      </c>
       <c r="L30" s="4">
         <f>IF(COUNT(H30:K30)=4,SUM(H30:K30),"")</f>
         <v/>
@@ -2037,21 +2359,59 @@
         <f>IF(OR(E30="",L30=""),"",IF(AND(L30&gt;=VLOOKUP(E30,Tiers!$A$4:$C$7,2,0),L30&lt;=VLOOKUP(E30,Tiers!$A$4:$C$7,3,0)),"OK","Fora"))</f>
         <v/>
       </c>
-      <c r="N30" s="5" t="n"/>
-      <c r="O30" s="5" t="n"/>
+      <c r="N30" s="5" t="inlineStr">
+        <is>
+          <t>Ganhar de NPC</t>
+        </is>
+      </c>
+      <c r="O30" s="5" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="inlineStr"/>
-      <c r="B31" s="5" t="inlineStr"/>
-      <c r="C31" s="5" t="inlineStr"/>
-      <c r="D31" s="5" t="inlineStr"/>
-      <c r="E31" s="4" t="inlineStr"/>
-      <c r="F31" s="4" t="inlineStr"/>
-      <c r="G31" s="5" t="inlineStr"/>
-      <c r="H31" s="4" t="inlineStr"/>
-      <c r="I31" s="4" t="inlineStr"/>
-      <c r="J31" s="4" t="inlineStr"/>
-      <c r="K31" s="4" t="inlineStr"/>
+      <c r="A31" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Sam</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>Sam</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>Aldeão</t>
+        </is>
+      </c>
+      <c r="E31" s="11" t="inlineStr">
+        <is>
+          <t>Incomum</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>Nenhum</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t>Villager:Sam</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I31" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="J31" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="K31" s="4" t="n">
+        <v>4</v>
+      </c>
       <c r="L31" s="4">
         <f>IF(COUNT(H31:K31)=4,SUM(H31:K31),"")</f>
         <v/>
@@ -2060,21 +2420,59 @@
         <f>IF(OR(E31="",L31=""),"",IF(AND(L31&gt;=VLOOKUP(E31,Tiers!$A$4:$C$7,2,0),L31&lt;=VLOOKUP(E31,Tiers!$A$4:$C$7,3,0)),"OK","Fora"))</f>
         <v/>
       </c>
-      <c r="N31" s="5" t="n"/>
-      <c r="O31" s="5" t="n"/>
+      <c r="N31" s="5" t="inlineStr">
+        <is>
+          <t>Ganhar de NPC</t>
+        </is>
+      </c>
+      <c r="O31" s="5" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="inlineStr"/>
-      <c r="B32" s="5" t="inlineStr"/>
-      <c r="C32" s="5" t="inlineStr"/>
-      <c r="D32" s="5" t="inlineStr"/>
-      <c r="E32" s="4" t="inlineStr"/>
-      <c r="F32" s="4" t="inlineStr"/>
-      <c r="G32" s="5" t="inlineStr"/>
-      <c r="H32" s="4" t="inlineStr"/>
-      <c r="I32" s="4" t="inlineStr"/>
-      <c r="J32" s="4" t="inlineStr"/>
-      <c r="K32" s="4" t="inlineStr"/>
+      <c r="A32" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Penny</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Penny</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Aldeão</t>
+        </is>
+      </c>
+      <c r="E32" s="11" t="inlineStr">
+        <is>
+          <t>Incomum</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>Nenhum</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>Villager:Penny</t>
+        </is>
+      </c>
+      <c r="H32" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="I32" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J32" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="K32" s="4" t="n">
+        <v>4</v>
+      </c>
       <c r="L32" s="4">
         <f>IF(COUNT(H32:K32)=4,SUM(H32:K32),"")</f>
         <v/>
@@ -2083,21 +2481,59 @@
         <f>IF(OR(E32="",L32=""),"",IF(AND(L32&gt;=VLOOKUP(E32,Tiers!$A$4:$C$7,2,0),L32&lt;=VLOOKUP(E32,Tiers!$A$4:$C$7,3,0)),"OK","Fora"))</f>
         <v/>
       </c>
-      <c r="N32" s="5" t="n"/>
-      <c r="O32" s="5" t="n"/>
+      <c r="N32" s="5" t="inlineStr">
+        <is>
+          <t>Ganhar de NPC</t>
+        </is>
+      </c>
+      <c r="O32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="inlineStr"/>
-      <c r="B33" s="5" t="inlineStr"/>
-      <c r="C33" s="5" t="inlineStr"/>
-      <c r="D33" s="5" t="inlineStr"/>
-      <c r="E33" s="4" t="inlineStr"/>
-      <c r="F33" s="4" t="inlineStr"/>
-      <c r="G33" s="5" t="inlineStr"/>
-      <c r="H33" s="4" t="inlineStr"/>
-      <c r="I33" s="4" t="inlineStr"/>
-      <c r="J33" s="4" t="inlineStr"/>
-      <c r="K33" s="4" t="inlineStr"/>
+      <c r="A33" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>Leah</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>Leah</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>Aldeão</t>
+        </is>
+      </c>
+      <c r="E33" s="11" t="inlineStr">
+        <is>
+          <t>Incomum</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>Nenhum</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t>Villager:Leah</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I33" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="J33" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="K33" s="4" t="n">
+        <v>5</v>
+      </c>
       <c r="L33" s="4">
         <f>IF(COUNT(H33:K33)=4,SUM(H33:K33),"")</f>
         <v/>
@@ -2106,21 +2542,59 @@
         <f>IF(OR(E33="",L33=""),"",IF(AND(L33&gt;=VLOOKUP(E33,Tiers!$A$4:$C$7,2,0),L33&lt;=VLOOKUP(E33,Tiers!$A$4:$C$7,3,0)),"OK","Fora"))</f>
         <v/>
       </c>
-      <c r="N33" s="5" t="n"/>
-      <c r="O33" s="5" t="n"/>
+      <c r="N33" s="5" t="inlineStr">
+        <is>
+          <t>Ganhar de NPC</t>
+        </is>
+      </c>
+      <c r="O33" s="5" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="4" t="inlineStr"/>
-      <c r="B34" s="5" t="inlineStr"/>
-      <c r="C34" s="5" t="inlineStr"/>
-      <c r="D34" s="5" t="inlineStr"/>
-      <c r="E34" s="4" t="inlineStr"/>
-      <c r="F34" s="4" t="inlineStr"/>
-      <c r="G34" s="5" t="inlineStr"/>
-      <c r="H34" s="4" t="inlineStr"/>
-      <c r="I34" s="4" t="inlineStr"/>
-      <c r="J34" s="4" t="inlineStr"/>
-      <c r="K34" s="4" t="inlineStr"/>
+      <c r="A34" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Elliott</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>Elliott</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Aldeão</t>
+        </is>
+      </c>
+      <c r="E34" s="11" t="inlineStr">
+        <is>
+          <t>Incomum</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>Nenhum</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>Villager:Elliott</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="I34" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="J34" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="K34" s="4" t="n">
+        <v>5</v>
+      </c>
       <c r="L34" s="4">
         <f>IF(COUNT(H34:K34)=4,SUM(H34:K34),"")</f>
         <v/>
@@ -2129,21 +2603,59 @@
         <f>IF(OR(E34="",L34=""),"",IF(AND(L34&gt;=VLOOKUP(E34,Tiers!$A$4:$C$7,2,0),L34&lt;=VLOOKUP(E34,Tiers!$A$4:$C$7,3,0)),"OK","Fora"))</f>
         <v/>
       </c>
-      <c r="N34" s="5" t="n"/>
-      <c r="O34" s="5" t="n"/>
+      <c r="N34" s="5" t="inlineStr">
+        <is>
+          <t>Ganhar de NPC</t>
+        </is>
+      </c>
+      <c r="O34" s="5" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="4" t="inlineStr"/>
-      <c r="B35" s="5" t="inlineStr"/>
-      <c r="C35" s="5" t="inlineStr"/>
-      <c r="D35" s="5" t="inlineStr"/>
-      <c r="E35" s="4" t="inlineStr"/>
-      <c r="F35" s="4" t="inlineStr"/>
-      <c r="G35" s="5" t="inlineStr"/>
-      <c r="H35" s="4" t="inlineStr"/>
-      <c r="I35" s="4" t="inlineStr"/>
-      <c r="J35" s="4" t="inlineStr"/>
-      <c r="K35" s="4" t="inlineStr"/>
+      <c r="A35" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Haley</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>Haley</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>Aldeão</t>
+        </is>
+      </c>
+      <c r="E35" s="11" t="inlineStr">
+        <is>
+          <t>Incomum</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>Nenhum</t>
+        </is>
+      </c>
+      <c r="G35" s="5" t="inlineStr">
+        <is>
+          <t>Villager:Haley</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="I35" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="J35" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="K35" s="4" t="n">
+        <v>4</v>
+      </c>
       <c r="L35" s="4">
         <f>IF(COUNT(H35:K35)=4,SUM(H35:K35),"")</f>
         <v/>
@@ -2152,21 +2664,59 @@
         <f>IF(OR(E35="",L35=""),"",IF(AND(L35&gt;=VLOOKUP(E35,Tiers!$A$4:$C$7,2,0),L35&lt;=VLOOKUP(E35,Tiers!$A$4:$C$7,3,0)),"OK","Fora"))</f>
         <v/>
       </c>
-      <c r="N35" s="5" t="n"/>
-      <c r="O35" s="5" t="n"/>
+      <c r="N35" s="5" t="inlineStr">
+        <is>
+          <t>Ganhar de NPC</t>
+        </is>
+      </c>
+      <c r="O35" s="5" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="4" t="inlineStr"/>
-      <c r="B36" s="5" t="inlineStr"/>
-      <c r="C36" s="5" t="inlineStr"/>
-      <c r="D36" s="5" t="inlineStr"/>
-      <c r="E36" s="4" t="inlineStr"/>
-      <c r="F36" s="4" t="inlineStr"/>
-      <c r="G36" s="5" t="inlineStr"/>
-      <c r="H36" s="4" t="inlineStr"/>
-      <c r="I36" s="4" t="inlineStr"/>
-      <c r="J36" s="4" t="inlineStr"/>
-      <c r="K36" s="4" t="inlineStr"/>
+      <c r="A36" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Maru</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>Maru</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Aldeão</t>
+        </is>
+      </c>
+      <c r="E36" s="11" t="inlineStr">
+        <is>
+          <t>Incomum</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>Nenhum</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>Villager:Maru</t>
+        </is>
+      </c>
+      <c r="H36" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I36" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J36" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="K36" s="4" t="n">
+        <v>5</v>
+      </c>
       <c r="L36" s="4">
         <f>IF(COUNT(H36:K36)=4,SUM(H36:K36),"")</f>
         <v/>
@@ -2175,21 +2725,59 @@
         <f>IF(OR(E36="",L36=""),"",IF(AND(L36&gt;=VLOOKUP(E36,Tiers!$A$4:$C$7,2,0),L36&lt;=VLOOKUP(E36,Tiers!$A$4:$C$7,3,0)),"OK","Fora"))</f>
         <v/>
       </c>
-      <c r="N36" s="5" t="n"/>
-      <c r="O36" s="5" t="n"/>
+      <c r="N36" s="5" t="inlineStr">
+        <is>
+          <t>Ganhar de NPC</t>
+        </is>
+      </c>
+      <c r="O36" s="5" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="4" t="inlineStr"/>
-      <c r="B37" s="5" t="inlineStr"/>
-      <c r="C37" s="5" t="inlineStr"/>
-      <c r="D37" s="5" t="inlineStr"/>
-      <c r="E37" s="4" t="inlineStr"/>
-      <c r="F37" s="4" t="inlineStr"/>
-      <c r="G37" s="5" t="inlineStr"/>
-      <c r="H37" s="4" t="inlineStr"/>
-      <c r="I37" s="4" t="inlineStr"/>
-      <c r="J37" s="4" t="inlineStr"/>
-      <c r="K37" s="4" t="inlineStr"/>
+      <c r="A37" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Emily</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>Emily</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Aldeão</t>
+        </is>
+      </c>
+      <c r="E37" s="11" t="inlineStr">
+        <is>
+          <t>Incomum</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>Nenhum</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>Villager:Emily</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="I37" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J37" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="K37" s="4" t="n">
+        <v>5</v>
+      </c>
       <c r="L37" s="4">
         <f>IF(COUNT(H37:K37)=4,SUM(H37:K37),"")</f>
         <v/>
@@ -2198,21 +2786,59 @@
         <f>IF(OR(E37="",L37=""),"",IF(AND(L37&gt;=VLOOKUP(E37,Tiers!$A$4:$C$7,2,0),L37&lt;=VLOOKUP(E37,Tiers!$A$4:$C$7,3,0)),"OK","Fora"))</f>
         <v/>
       </c>
-      <c r="N37" s="5" t="n"/>
-      <c r="O37" s="5" t="n"/>
+      <c r="N37" s="5" t="inlineStr">
+        <is>
+          <t>Ganhar de NPC</t>
+        </is>
+      </c>
+      <c r="O37" s="5" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="4" t="inlineStr"/>
-      <c r="B38" s="5" t="inlineStr"/>
-      <c r="C38" s="5" t="inlineStr"/>
-      <c r="D38" s="5" t="inlineStr"/>
-      <c r="E38" s="4" t="inlineStr"/>
-      <c r="F38" s="4" t="inlineStr"/>
-      <c r="G38" s="5" t="inlineStr"/>
-      <c r="H38" s="4" t="inlineStr"/>
-      <c r="I38" s="4" t="inlineStr"/>
-      <c r="J38" s="4" t="inlineStr"/>
-      <c r="K38" s="4" t="inlineStr"/>
+      <c r="A38" s="4" t="n">
+        <v>34</v>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>Shane</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>Shane</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Aldeão</t>
+        </is>
+      </c>
+      <c r="E38" s="11" t="inlineStr">
+        <is>
+          <t>Incomum</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>Nenhum</t>
+        </is>
+      </c>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>Villager:Shane</t>
+        </is>
+      </c>
+      <c r="H38" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="I38" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="J38" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="K38" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="L38" s="4">
         <f>IF(COUNT(H38:K38)=4,SUM(H38:K38),"")</f>
         <v/>
@@ -2221,21 +2847,59 @@
         <f>IF(OR(E38="",L38=""),"",IF(AND(L38&gt;=VLOOKUP(E38,Tiers!$A$4:$C$7,2,0),L38&lt;=VLOOKUP(E38,Tiers!$A$4:$C$7,3,0)),"OK","Fora"))</f>
         <v/>
       </c>
-      <c r="N38" s="5" t="n"/>
-      <c r="O38" s="5" t="n"/>
+      <c r="N38" s="5" t="inlineStr">
+        <is>
+          <t>Ganhar de NPC</t>
+        </is>
+      </c>
+      <c r="O38" s="5" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="4" t="inlineStr"/>
-      <c r="B39" s="5" t="inlineStr"/>
-      <c r="C39" s="5" t="inlineStr"/>
-      <c r="D39" s="5" t="inlineStr"/>
-      <c r="E39" s="4" t="inlineStr"/>
-      <c r="F39" s="4" t="inlineStr"/>
-      <c r="G39" s="5" t="inlineStr"/>
-      <c r="H39" s="4" t="inlineStr"/>
-      <c r="I39" s="4" t="inlineStr"/>
-      <c r="J39" s="4" t="inlineStr"/>
-      <c r="K39" s="4" t="inlineStr"/>
+      <c r="A39" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>Gus</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>Gus</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Aldeão</t>
+        </is>
+      </c>
+      <c r="E39" s="11" t="inlineStr">
+        <is>
+          <t>Incomum</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>Nenhum</t>
+        </is>
+      </c>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>Villager:Gus</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="I39" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J39" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="K39" s="4" t="n">
+        <v>5</v>
+      </c>
       <c r="L39" s="4">
         <f>IF(COUNT(H39:K39)=4,SUM(H39:K39),"")</f>
         <v/>
@@ -2244,21 +2908,63 @@
         <f>IF(OR(E39="",L39=""),"",IF(AND(L39&gt;=VLOOKUP(E39,Tiers!$A$4:$C$7,2,0),L39&lt;=VLOOKUP(E39,Tiers!$A$4:$C$7,3,0)),"OK","Fora"))</f>
         <v/>
       </c>
-      <c r="N39" s="5" t="n"/>
-      <c r="O39" s="5" t="n"/>
+      <c r="N39" s="5" t="inlineStr">
+        <is>
+          <t>Ganhar de NPC</t>
+        </is>
+      </c>
+      <c r="O39" s="5" t="inlineStr">
+        <is>
+          <t>dono do Saloon</t>
+        </is>
+      </c>
     </row>
     <row r="40">
-      <c r="A40" s="4" t="inlineStr"/>
-      <c r="B40" s="5" t="inlineStr"/>
-      <c r="C40" s="5" t="inlineStr"/>
-      <c r="D40" s="5" t="inlineStr"/>
-      <c r="E40" s="4" t="inlineStr"/>
-      <c r="F40" s="4" t="inlineStr"/>
-      <c r="G40" s="5" t="inlineStr"/>
-      <c r="H40" s="4" t="inlineStr"/>
-      <c r="I40" s="4" t="inlineStr"/>
-      <c r="J40" s="4" t="inlineStr"/>
-      <c r="K40" s="4" t="inlineStr"/>
+      <c r="A40" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>Pierre</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>Pierre</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Aldeão</t>
+        </is>
+      </c>
+      <c r="E40" s="11" t="inlineStr">
+        <is>
+          <t>Incomum</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>Nenhum</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>Villager:Pierre</t>
+        </is>
+      </c>
+      <c r="H40" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I40" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="J40" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="K40" s="4" t="n">
+        <v>4</v>
+      </c>
       <c r="L40" s="4">
         <f>IF(COUNT(H40:K40)=4,SUM(H40:K40),"")</f>
         <v/>
@@ -2267,21 +2973,59 @@
         <f>IF(OR(E40="",L40=""),"",IF(AND(L40&gt;=VLOOKUP(E40,Tiers!$A$4:$C$7,2,0),L40&lt;=VLOOKUP(E40,Tiers!$A$4:$C$7,3,0)),"OK","Fora"))</f>
         <v/>
       </c>
-      <c r="N40" s="5" t="n"/>
-      <c r="O40" s="5" t="n"/>
+      <c r="N40" s="5" t="inlineStr">
+        <is>
+          <t>Ganhar de NPC</t>
+        </is>
+      </c>
+      <c r="O40" s="5" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="4" t="inlineStr"/>
-      <c r="B41" s="5" t="inlineStr"/>
-      <c r="C41" s="5" t="inlineStr"/>
-      <c r="D41" s="5" t="inlineStr"/>
-      <c r="E41" s="4" t="inlineStr"/>
-      <c r="F41" s="4" t="inlineStr"/>
-      <c r="G41" s="5" t="inlineStr"/>
-      <c r="H41" s="4" t="inlineStr"/>
-      <c r="I41" s="4" t="inlineStr"/>
-      <c r="J41" s="4" t="inlineStr"/>
-      <c r="K41" s="4" t="inlineStr"/>
+      <c r="A41" s="4" t="n">
+        <v>37</v>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>Robin</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>Robin</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Aldeão</t>
+        </is>
+      </c>
+      <c r="E41" s="11" t="inlineStr">
+        <is>
+          <t>Incomum</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>Nenhum</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>Villager:Robin</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I41" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J41" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="K41" s="4" t="n">
+        <v>4</v>
+      </c>
       <c r="L41" s="4">
         <f>IF(COUNT(H41:K41)=4,SUM(H41:K41),"")</f>
         <v/>
@@ -2290,21 +3034,59 @@
         <f>IF(OR(E41="",L41=""),"",IF(AND(L41&gt;=VLOOKUP(E41,Tiers!$A$4:$C$7,2,0),L41&lt;=VLOOKUP(E41,Tiers!$A$4:$C$7,3,0)),"OK","Fora"))</f>
         <v/>
       </c>
-      <c r="N41" s="5" t="n"/>
-      <c r="O41" s="5" t="n"/>
+      <c r="N41" s="5" t="inlineStr">
+        <is>
+          <t>Ganhar de NPC</t>
+        </is>
+      </c>
+      <c r="O41" s="5" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" s="4" t="inlineStr"/>
-      <c r="B42" s="5" t="inlineStr"/>
-      <c r="C42" s="5" t="inlineStr"/>
-      <c r="D42" s="5" t="inlineStr"/>
-      <c r="E42" s="4" t="inlineStr"/>
-      <c r="F42" s="4" t="inlineStr"/>
-      <c r="G42" s="5" t="inlineStr"/>
-      <c r="H42" s="4" t="inlineStr"/>
-      <c r="I42" s="4" t="inlineStr"/>
-      <c r="J42" s="4" t="inlineStr"/>
-      <c r="K42" s="4" t="inlineStr"/>
+      <c r="A42" s="4" t="n">
+        <v>38</v>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>Clint</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>Clint</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Aldeão</t>
+        </is>
+      </c>
+      <c r="E42" s="11" t="inlineStr">
+        <is>
+          <t>Incomum</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>Nenhum</t>
+        </is>
+      </c>
+      <c r="G42" s="5" t="inlineStr">
+        <is>
+          <t>Villager:Clint</t>
+        </is>
+      </c>
+      <c r="H42" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="I42" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="J42" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="K42" s="4" t="n">
+        <v>4</v>
+      </c>
       <c r="L42" s="4">
         <f>IF(COUNT(H42:K42)=4,SUM(H42:K42),"")</f>
         <v/>
@@ -2313,21 +3095,59 @@
         <f>IF(OR(E42="",L42=""),"",IF(AND(L42&gt;=VLOOKUP(E42,Tiers!$A$4:$C$7,2,0),L42&lt;=VLOOKUP(E42,Tiers!$A$4:$C$7,3,0)),"OK","Fora"))</f>
         <v/>
       </c>
-      <c r="N42" s="5" t="n"/>
-      <c r="O42" s="5" t="n"/>
+      <c r="N42" s="5" t="inlineStr">
+        <is>
+          <t>Ganhar de NPC</t>
+        </is>
+      </c>
+      <c r="O42" s="5" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="4" t="inlineStr"/>
-      <c r="B43" s="5" t="inlineStr"/>
-      <c r="C43" s="5" t="inlineStr"/>
-      <c r="D43" s="5" t="inlineStr"/>
-      <c r="E43" s="4" t="inlineStr"/>
-      <c r="F43" s="4" t="inlineStr"/>
-      <c r="G43" s="5" t="inlineStr"/>
-      <c r="H43" s="4" t="inlineStr"/>
-      <c r="I43" s="4" t="inlineStr"/>
-      <c r="J43" s="4" t="inlineStr"/>
-      <c r="K43" s="4" t="inlineStr"/>
+      <c r="A43" s="4" t="n">
+        <v>39</v>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>Willy</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>Willy</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>Aldeão</t>
+        </is>
+      </c>
+      <c r="E43" s="11" t="inlineStr">
+        <is>
+          <t>Incomum</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>Nenhum</t>
+        </is>
+      </c>
+      <c r="G43" s="5" t="inlineStr">
+        <is>
+          <t>Villager:Willy</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="I43" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J43" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="K43" s="4" t="n">
+        <v>4</v>
+      </c>
       <c r="L43" s="4">
         <f>IF(COUNT(H43:K43)=4,SUM(H43:K43),"")</f>
         <v/>
@@ -2336,21 +3156,59 @@
         <f>IF(OR(E43="",L43=""),"",IF(AND(L43&gt;=VLOOKUP(E43,Tiers!$A$4:$C$7,2,0),L43&lt;=VLOOKUP(E43,Tiers!$A$4:$C$7,3,0)),"OK","Fora"))</f>
         <v/>
       </c>
-      <c r="N43" s="5" t="n"/>
-      <c r="O43" s="5" t="n"/>
+      <c r="N43" s="5" t="inlineStr">
+        <is>
+          <t>Ganhar de NPC</t>
+        </is>
+      </c>
+      <c r="O43" s="5" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="4" t="inlineStr"/>
-      <c r="B44" s="5" t="inlineStr"/>
-      <c r="C44" s="5" t="inlineStr"/>
-      <c r="D44" s="5" t="inlineStr"/>
-      <c r="E44" s="4" t="inlineStr"/>
-      <c r="F44" s="4" t="inlineStr"/>
-      <c r="G44" s="5" t="inlineStr"/>
-      <c r="H44" s="4" t="inlineStr"/>
-      <c r="I44" s="4" t="inlineStr"/>
-      <c r="J44" s="4" t="inlineStr"/>
-      <c r="K44" s="4" t="inlineStr"/>
+      <c r="A44" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>Skeleton</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>Esqueleto</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Monstro</t>
+        </is>
+      </c>
+      <c r="E44" s="12" t="inlineStr">
+        <is>
+          <t>Raro</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>Nenhum</t>
+        </is>
+      </c>
+      <c r="G44" s="5" t="inlineStr">
+        <is>
+          <t>Monster:Skeleton</t>
+        </is>
+      </c>
+      <c r="H44" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="I44" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="J44" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="K44" s="4" t="n">
+        <v>6</v>
+      </c>
       <c r="L44" s="4">
         <f>IF(COUNT(H44:K44)=4,SUM(H44:K44),"")</f>
         <v/>
@@ -2359,21 +3217,59 @@
         <f>IF(OR(E44="",L44=""),"",IF(AND(L44&gt;=VLOOKUP(E44,Tiers!$A$4:$C$7,2,0),L44&lt;=VLOOKUP(E44,Tiers!$A$4:$C$7,3,0)),"OK","Fora"))</f>
         <v/>
       </c>
-      <c r="N44" s="5" t="n"/>
-      <c r="O44" s="5" t="n"/>
+      <c r="N44" s="5" t="inlineStr">
+        <is>
+          <t>Ganhar de NPC</t>
+        </is>
+      </c>
+      <c r="O44" s="5" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="4" t="inlineStr"/>
-      <c r="B45" s="5" t="inlineStr"/>
-      <c r="C45" s="5" t="inlineStr"/>
-      <c r="D45" s="5" t="inlineStr"/>
-      <c r="E45" s="4" t="inlineStr"/>
-      <c r="F45" s="4" t="inlineStr"/>
-      <c r="G45" s="5" t="inlineStr"/>
-      <c r="H45" s="4" t="inlineStr"/>
-      <c r="I45" s="4" t="inlineStr"/>
-      <c r="J45" s="4" t="inlineStr"/>
-      <c r="K45" s="4" t="inlineStr"/>
+      <c r="A45" s="4" t="n">
+        <v>41</v>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>Shadow Brute</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>Bruto das Sombras</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Monstro</t>
+        </is>
+      </c>
+      <c r="E45" s="12" t="inlineStr">
+        <is>
+          <t>Raro</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>Nenhum</t>
+        </is>
+      </c>
+      <c r="G45" s="5" t="inlineStr">
+        <is>
+          <t>Monster:ShadowBrute</t>
+        </is>
+      </c>
+      <c r="H45" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="I45" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="J45" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="K45" s="4" t="n">
+        <v>5</v>
+      </c>
       <c r="L45" s="4">
         <f>IF(COUNT(H45:K45)=4,SUM(H45:K45),"")</f>
         <v/>
@@ -2382,21 +3278,59 @@
         <f>IF(OR(E45="",L45=""),"",IF(AND(L45&gt;=VLOOKUP(E45,Tiers!$A$4:$C$7,2,0),L45&lt;=VLOOKUP(E45,Tiers!$A$4:$C$7,3,0)),"OK","Fora"))</f>
         <v/>
       </c>
-      <c r="N45" s="5" t="n"/>
-      <c r="O45" s="5" t="n"/>
+      <c r="N45" s="5" t="inlineStr">
+        <is>
+          <t>Ganhar de NPC</t>
+        </is>
+      </c>
+      <c r="O45" s="5" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="4" t="inlineStr"/>
-      <c r="B46" s="5" t="inlineStr"/>
-      <c r="C46" s="5" t="inlineStr"/>
-      <c r="D46" s="5" t="inlineStr"/>
-      <c r="E46" s="4" t="inlineStr"/>
-      <c r="F46" s="4" t="inlineStr"/>
-      <c r="G46" s="5" t="inlineStr"/>
-      <c r="H46" s="4" t="inlineStr"/>
-      <c r="I46" s="4" t="inlineStr"/>
-      <c r="J46" s="4" t="inlineStr"/>
-      <c r="K46" s="4" t="inlineStr"/>
+      <c r="A46" s="4" t="n">
+        <v>42</v>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>Serpent</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>Serpente</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Monstro</t>
+        </is>
+      </c>
+      <c r="E46" s="12" t="inlineStr">
+        <is>
+          <t>Raro</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>Nenhum</t>
+        </is>
+      </c>
+      <c r="G46" s="5" t="inlineStr">
+        <is>
+          <t>Monster:Serpent</t>
+        </is>
+      </c>
+      <c r="H46" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="I46" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="J46" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="K46" s="4" t="n">
+        <v>5</v>
+      </c>
       <c r="L46" s="4">
         <f>IF(COUNT(H46:K46)=4,SUM(H46:K46),"")</f>
         <v/>
@@ -2405,21 +3339,59 @@
         <f>IF(OR(E46="",L46=""),"",IF(AND(L46&gt;=VLOOKUP(E46,Tiers!$A$4:$C$7,2,0),L46&lt;=VLOOKUP(E46,Tiers!$A$4:$C$7,3,0)),"OK","Fora"))</f>
         <v/>
       </c>
-      <c r="N46" s="5" t="n"/>
-      <c r="O46" s="5" t="n"/>
+      <c r="N46" s="5" t="inlineStr">
+        <is>
+          <t>Ganhar de NPC</t>
+        </is>
+      </c>
+      <c r="O46" s="5" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="4" t="inlineStr"/>
-      <c r="B47" s="5" t="inlineStr"/>
-      <c r="C47" s="5" t="inlineStr"/>
-      <c r="D47" s="5" t="inlineStr"/>
-      <c r="E47" s="4" t="inlineStr"/>
-      <c r="F47" s="4" t="inlineStr"/>
-      <c r="G47" s="5" t="inlineStr"/>
-      <c r="H47" s="4" t="inlineStr"/>
-      <c r="I47" s="4" t="inlineStr"/>
-      <c r="J47" s="4" t="inlineStr"/>
-      <c r="K47" s="4" t="inlineStr"/>
+      <c r="A47" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>Pepper Rex</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>Pepper Rex</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>Monstro</t>
+        </is>
+      </c>
+      <c r="E47" s="12" t="inlineStr">
+        <is>
+          <t>Raro</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>Nenhum</t>
+        </is>
+      </c>
+      <c r="G47" s="5" t="inlineStr">
+        <is>
+          <t>Monster:PepperRex</t>
+        </is>
+      </c>
+      <c r="H47" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="I47" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="J47" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="K47" s="4" t="n">
+        <v>6</v>
+      </c>
       <c r="L47" s="4">
         <f>IF(COUNT(H47:K47)=4,SUM(H47:K47),"")</f>
         <v/>
@@ -2428,21 +3400,63 @@
         <f>IF(OR(E47="",L47=""),"",IF(AND(L47&gt;=VLOOKUP(E47,Tiers!$A$4:$C$7,2,0),L47&lt;=VLOOKUP(E47,Tiers!$A$4:$C$7,3,0)),"OK","Fora"))</f>
         <v/>
       </c>
-      <c r="N47" s="5" t="n"/>
-      <c r="O47" s="5" t="n"/>
+      <c r="N47" s="5" t="inlineStr">
+        <is>
+          <t>Ganhar de NPC</t>
+        </is>
+      </c>
+      <c r="O47" s="5" t="inlineStr">
+        <is>
+          <t>dino das cavernas</t>
+        </is>
+      </c>
     </row>
     <row r="48">
-      <c r="A48" s="4" t="inlineStr"/>
-      <c r="B48" s="5" t="inlineStr"/>
-      <c r="C48" s="5" t="inlineStr"/>
-      <c r="D48" s="5" t="inlineStr"/>
-      <c r="E48" s="4" t="inlineStr"/>
-      <c r="F48" s="4" t="inlineStr"/>
-      <c r="G48" s="5" t="inlineStr"/>
-      <c r="H48" s="4" t="inlineStr"/>
-      <c r="I48" s="4" t="inlineStr"/>
-      <c r="J48" s="4" t="inlineStr"/>
-      <c r="K48" s="4" t="inlineStr"/>
+      <c r="A48" s="4" t="n">
+        <v>44</v>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>Diamond</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>Diamante</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Mineral</t>
+        </is>
+      </c>
+      <c r="E48" s="12" t="inlineStr">
+        <is>
+          <t>Raro</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>Nenhum</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr">
+        <is>
+          <t>(O)72</t>
+        </is>
+      </c>
+      <c r="H48" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="I48" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="J48" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="K48" s="4" t="n">
+        <v>6</v>
+      </c>
       <c r="L48" s="4">
         <f>IF(COUNT(H48:K48)=4,SUM(H48:K48),"")</f>
         <v/>
@@ -2451,21 +3465,59 @@
         <f>IF(OR(E48="",L48=""),"",IF(AND(L48&gt;=VLOOKUP(E48,Tiers!$A$4:$C$7,2,0),L48&lt;=VLOOKUP(E48,Tiers!$A$4:$C$7,3,0)),"OK","Fora"))</f>
         <v/>
       </c>
-      <c r="N48" s="5" t="n"/>
-      <c r="O48" s="5" t="n"/>
+      <c r="N48" s="5" t="inlineStr">
+        <is>
+          <t>Ganhar de NPC</t>
+        </is>
+      </c>
+      <c r="O48" s="5" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="4" t="inlineStr"/>
-      <c r="B49" s="5" t="inlineStr"/>
-      <c r="C49" s="5" t="inlineStr"/>
-      <c r="D49" s="5" t="inlineStr"/>
-      <c r="E49" s="4" t="inlineStr"/>
-      <c r="F49" s="4" t="inlineStr"/>
-      <c r="G49" s="5" t="inlineStr"/>
-      <c r="H49" s="4" t="inlineStr"/>
-      <c r="I49" s="4" t="inlineStr"/>
-      <c r="J49" s="4" t="inlineStr"/>
-      <c r="K49" s="4" t="inlineStr"/>
+      <c r="A49" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>Ancient Fruit</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>Fruta Ancestral</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>Crop</t>
+        </is>
+      </c>
+      <c r="E49" s="12" t="inlineStr">
+        <is>
+          <t>Raro</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>Nenhum</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr">
+        <is>
+          <t>(O)454</t>
+        </is>
+      </c>
+      <c r="H49" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="I49" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="J49" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="K49" s="4" t="n">
+        <v>6</v>
+      </c>
       <c r="L49" s="4">
         <f>IF(COUNT(H49:K49)=4,SUM(H49:K49),"")</f>
         <v/>
@@ -2474,21 +3526,59 @@
         <f>IF(OR(E49="",L49=""),"",IF(AND(L49&gt;=VLOOKUP(E49,Tiers!$A$4:$C$7,2,0),L49&lt;=VLOOKUP(E49,Tiers!$A$4:$C$7,3,0)),"OK","Fora"))</f>
         <v/>
       </c>
-      <c r="N49" s="5" t="n"/>
-      <c r="O49" s="5" t="n"/>
+      <c r="N49" s="5" t="inlineStr">
+        <is>
+          <t>Ganhar de NPC</t>
+        </is>
+      </c>
+      <c r="O49" s="5" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="4" t="inlineStr"/>
-      <c r="B50" s="5" t="inlineStr"/>
-      <c r="C50" s="5" t="inlineStr"/>
-      <c r="D50" s="5" t="inlineStr"/>
-      <c r="E50" s="4" t="inlineStr"/>
-      <c r="F50" s="4" t="inlineStr"/>
-      <c r="G50" s="5" t="inlineStr"/>
-      <c r="H50" s="4" t="inlineStr"/>
-      <c r="I50" s="4" t="inlineStr"/>
-      <c r="J50" s="4" t="inlineStr"/>
-      <c r="K50" s="4" t="inlineStr"/>
+      <c r="A50" s="4" t="n">
+        <v>46</v>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>Sturgeon</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>Esturjão</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Peixe</t>
+        </is>
+      </c>
+      <c r="E50" s="12" t="inlineStr">
+        <is>
+          <t>Raro</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t>Nenhum</t>
+        </is>
+      </c>
+      <c r="G50" s="5" t="inlineStr">
+        <is>
+          <t>(O)698</t>
+        </is>
+      </c>
+      <c r="H50" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="I50" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="J50" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="K50" s="4" t="n">
+        <v>5</v>
+      </c>
       <c r="L50" s="4">
         <f>IF(COUNT(H50:K50)=4,SUM(H50:K50),"")</f>
         <v/>
@@ -2497,21 +3587,59 @@
         <f>IF(OR(E50="",L50=""),"",IF(AND(L50&gt;=VLOOKUP(E50,Tiers!$A$4:$C$7,2,0),L50&lt;=VLOOKUP(E50,Tiers!$A$4:$C$7,3,0)),"OK","Fora"))</f>
         <v/>
       </c>
-      <c r="N50" s="5" t="n"/>
-      <c r="O50" s="5" t="n"/>
+      <c r="N50" s="5" t="inlineStr">
+        <is>
+          <t>Ganhar de NPC</t>
+        </is>
+      </c>
+      <c r="O50" s="5" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="4" t="inlineStr"/>
-      <c r="B51" s="5" t="inlineStr"/>
-      <c r="C51" s="5" t="inlineStr"/>
-      <c r="D51" s="5" t="inlineStr"/>
-      <c r="E51" s="4" t="inlineStr"/>
-      <c r="F51" s="4" t="inlineStr"/>
-      <c r="G51" s="5" t="inlineStr"/>
-      <c r="H51" s="4" t="inlineStr"/>
-      <c r="I51" s="4" t="inlineStr"/>
-      <c r="J51" s="4" t="inlineStr"/>
-      <c r="K51" s="4" t="inlineStr"/>
+      <c r="A51" s="4" t="n">
+        <v>47</v>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>Sweet Gem Berry</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>Baga-joia Doce</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>Crop</t>
+        </is>
+      </c>
+      <c r="E51" s="12" t="inlineStr">
+        <is>
+          <t>Raro</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>Nenhum</t>
+        </is>
+      </c>
+      <c r="G51" s="5" t="inlineStr">
+        <is>
+          <t>(O)417</t>
+        </is>
+      </c>
+      <c r="H51" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="I51" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="J51" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="K51" s="4" t="n">
+        <v>6</v>
+      </c>
       <c r="L51" s="4">
         <f>IF(COUNT(H51:K51)=4,SUM(H51:K51),"")</f>
         <v/>
@@ -2520,21 +3648,59 @@
         <f>IF(OR(E51="",L51=""),"",IF(AND(L51&gt;=VLOOKUP(E51,Tiers!$A$4:$C$7,2,0),L51&lt;=VLOOKUP(E51,Tiers!$A$4:$C$7,3,0)),"OK","Fora"))</f>
         <v/>
       </c>
-      <c r="N51" s="5" t="n"/>
-      <c r="O51" s="5" t="n"/>
+      <c r="N51" s="5" t="inlineStr">
+        <is>
+          <t>Ganhar de NPC</t>
+        </is>
+      </c>
+      <c r="O51" s="5" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" s="4" t="inlineStr"/>
-      <c r="B52" s="5" t="inlineStr"/>
-      <c r="C52" s="5" t="inlineStr"/>
-      <c r="D52" s="5" t="inlineStr"/>
-      <c r="E52" s="4" t="inlineStr"/>
-      <c r="F52" s="4" t="inlineStr"/>
-      <c r="G52" s="5" t="inlineStr"/>
-      <c r="H52" s="4" t="inlineStr"/>
-      <c r="I52" s="4" t="inlineStr"/>
-      <c r="J52" s="4" t="inlineStr"/>
-      <c r="K52" s="4" t="inlineStr"/>
+      <c r="A52" s="4" t="n">
+        <v>48</v>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>Wizard</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>Mago</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Aldeão</t>
+        </is>
+      </c>
+      <c r="E52" s="13" t="inlineStr">
+        <is>
+          <t>Lendário</t>
+        </is>
+      </c>
+      <c r="F52" s="4" t="inlineStr">
+        <is>
+          <t>Nenhum</t>
+        </is>
+      </c>
+      <c r="G52" s="5" t="inlineStr">
+        <is>
+          <t>Villager:Wizard</t>
+        </is>
+      </c>
+      <c r="H52" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="I52" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="J52" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="K52" s="4" t="n">
+        <v>8</v>
+      </c>
       <c r="L52" s="4">
         <f>IF(COUNT(H52:K52)=4,SUM(H52:K52),"")</f>
         <v/>
@@ -2543,21 +3709,63 @@
         <f>IF(OR(E52="",L52=""),"",IF(AND(L52&gt;=VLOOKUP(E52,Tiers!$A$4:$C$7,2,0),L52&lt;=VLOOKUP(E52,Tiers!$A$4:$C$7,3,0)),"OK","Fora"))</f>
         <v/>
       </c>
-      <c r="N52" s="5" t="n"/>
-      <c r="O52" s="5" t="n"/>
+      <c r="N52" s="5" t="inlineStr">
+        <is>
+          <t>Campeão</t>
+        </is>
+      </c>
+      <c r="O52" s="5" t="inlineStr">
+        <is>
+          <t>boss</t>
+        </is>
+      </c>
     </row>
     <row r="53">
-      <c r="A53" s="4" t="inlineStr"/>
-      <c r="B53" s="5" t="inlineStr"/>
-      <c r="C53" s="5" t="inlineStr"/>
-      <c r="D53" s="5" t="inlineStr"/>
-      <c r="E53" s="4" t="inlineStr"/>
-      <c r="F53" s="4" t="inlineStr"/>
-      <c r="G53" s="5" t="inlineStr"/>
-      <c r="H53" s="4" t="inlineStr"/>
-      <c r="I53" s="4" t="inlineStr"/>
-      <c r="J53" s="4" t="inlineStr"/>
-      <c r="K53" s="4" t="inlineStr"/>
+      <c r="A53" s="4" t="n">
+        <v>49</v>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>Junimo King</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>Rei Junimo</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>Especial</t>
+        </is>
+      </c>
+      <c r="E53" s="13" t="inlineStr">
+        <is>
+          <t>Lendário</t>
+        </is>
+      </c>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
+          <t>Nenhum</t>
+        </is>
+      </c>
+      <c r="G53" s="5" t="inlineStr">
+        <is>
+          <t>Special:JunimoKing</t>
+        </is>
+      </c>
+      <c r="H53" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="I53" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="J53" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="K53" s="4" t="n">
+        <v>9</v>
+      </c>
       <c r="L53" s="4">
         <f>IF(COUNT(H53:K53)=4,SUM(H53:K53),"")</f>
         <v/>
@@ -2566,21 +3774,63 @@
         <f>IF(OR(E53="",L53=""),"",IF(AND(L53&gt;=VLOOKUP(E53,Tiers!$A$4:$C$7,2,0),L53&lt;=VLOOKUP(E53,Tiers!$A$4:$C$7,3,0)),"OK","Fora"))</f>
         <v/>
       </c>
-      <c r="N53" s="5" t="n"/>
-      <c r="O53" s="5" t="n"/>
+      <c r="N53" s="5" t="inlineStr">
+        <is>
+          <t>Campeão</t>
+        </is>
+      </c>
+      <c r="O53" s="5" t="inlineStr">
+        <is>
+          <t>boss</t>
+        </is>
+      </c>
     </row>
     <row r="54">
-      <c r="A54" s="4" t="inlineStr"/>
-      <c r="B54" s="5" t="inlineStr"/>
-      <c r="C54" s="5" t="inlineStr"/>
-      <c r="D54" s="5" t="inlineStr"/>
-      <c r="E54" s="4" t="inlineStr"/>
-      <c r="F54" s="4" t="inlineStr"/>
-      <c r="G54" s="5" t="inlineStr"/>
-      <c r="H54" s="4" t="inlineStr"/>
-      <c r="I54" s="4" t="inlineStr"/>
-      <c r="J54" s="4" t="inlineStr"/>
-      <c r="K54" s="4" t="inlineStr"/>
+      <c r="A54" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>Mr. Qi</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>Sr. Qi</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>Especial</t>
+        </is>
+      </c>
+      <c r="E54" s="13" t="inlineStr">
+        <is>
+          <t>Lendário</t>
+        </is>
+      </c>
+      <c r="F54" s="4" t="inlineStr">
+        <is>
+          <t>Nenhum</t>
+        </is>
+      </c>
+      <c r="G54" s="5" t="inlineStr">
+        <is>
+          <t>Villager:Qi</t>
+        </is>
+      </c>
+      <c r="H54" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="I54" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="J54" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="K54" s="4" t="n">
+        <v>8</v>
+      </c>
       <c r="L54" s="4">
         <f>IF(COUNT(H54:K54)=4,SUM(H54:K54),"")</f>
         <v/>
@@ -2589,21 +3839,63 @@
         <f>IF(OR(E54="",L54=""),"",IF(AND(L54&gt;=VLOOKUP(E54,Tiers!$A$4:$C$7,2,0),L54&lt;=VLOOKUP(E54,Tiers!$A$4:$C$7,3,0)),"OK","Fora"))</f>
         <v/>
       </c>
-      <c r="N54" s="5" t="n"/>
-      <c r="O54" s="5" t="n"/>
+      <c r="N54" s="5" t="inlineStr">
+        <is>
+          <t>Campeão</t>
+        </is>
+      </c>
+      <c r="O54" s="5" t="inlineStr">
+        <is>
+          <t>boss</t>
+        </is>
+      </c>
     </row>
     <row r="55">
-      <c r="A55" s="4" t="inlineStr"/>
-      <c r="B55" s="5" t="inlineStr"/>
-      <c r="C55" s="5" t="inlineStr"/>
-      <c r="D55" s="5" t="inlineStr"/>
-      <c r="E55" s="4" t="inlineStr"/>
-      <c r="F55" s="4" t="inlineStr"/>
-      <c r="G55" s="5" t="inlineStr"/>
-      <c r="H55" s="4" t="inlineStr"/>
-      <c r="I55" s="4" t="inlineStr"/>
-      <c r="J55" s="4" t="inlineStr"/>
-      <c r="K55" s="4" t="inlineStr"/>
+      <c r="A55" s="4" t="n">
+        <v>51</v>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>Crimsonfish</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>Peixe Carmesim</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>Peixe</t>
+        </is>
+      </c>
+      <c r="E55" s="13" t="inlineStr">
+        <is>
+          <t>Lendário</t>
+        </is>
+      </c>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>Nenhum</t>
+        </is>
+      </c>
+      <c r="G55" s="5" t="inlineStr">
+        <is>
+          <t>(O)159</t>
+        </is>
+      </c>
+      <c r="H55" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="I55" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="J55" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="K55" s="4" t="n">
+        <v>6</v>
+      </c>
       <c r="L55" s="4">
         <f>IF(COUNT(H55:K55)=4,SUM(H55:K55),"")</f>
         <v/>
@@ -2612,21 +3904,63 @@
         <f>IF(OR(E55="",L55=""),"",IF(AND(L55&gt;=VLOOKUP(E55,Tiers!$A$4:$C$7,2,0),L55&lt;=VLOOKUP(E55,Tiers!$A$4:$C$7,3,0)),"OK","Fora"))</f>
         <v/>
       </c>
-      <c r="N55" s="5" t="n"/>
-      <c r="O55" s="5" t="n"/>
+      <c r="N55" s="5" t="inlineStr">
+        <is>
+          <t>Campeão</t>
+        </is>
+      </c>
+      <c r="O55" s="5" t="inlineStr">
+        <is>
+          <t>peixe lendário</t>
+        </is>
+      </c>
     </row>
     <row r="56">
-      <c r="A56" s="4" t="inlineStr"/>
-      <c r="B56" s="5" t="inlineStr"/>
-      <c r="C56" s="5" t="inlineStr"/>
-      <c r="D56" s="5" t="inlineStr"/>
-      <c r="E56" s="4" t="inlineStr"/>
-      <c r="F56" s="4" t="inlineStr"/>
-      <c r="G56" s="5" t="inlineStr"/>
-      <c r="H56" s="4" t="inlineStr"/>
-      <c r="I56" s="4" t="inlineStr"/>
-      <c r="J56" s="4" t="inlineStr"/>
-      <c r="K56" s="4" t="inlineStr"/>
+      <c r="A56" s="4" t="n">
+        <v>52</v>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>Prismatic Shard</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>Fragmento Prismático</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>Mineral</t>
+        </is>
+      </c>
+      <c r="E56" s="13" t="inlineStr">
+        <is>
+          <t>Lendário</t>
+        </is>
+      </c>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
+          <t>Nenhum</t>
+        </is>
+      </c>
+      <c r="G56" s="5" t="inlineStr">
+        <is>
+          <t>(O)74</t>
+        </is>
+      </c>
+      <c r="H56" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="I56" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="J56" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="K56" s="4" t="n">
+        <v>9</v>
+      </c>
       <c r="L56" s="4">
         <f>IF(COUNT(H56:K56)=4,SUM(H56:K56),"")</f>
         <v/>
@@ -2635,21 +3969,167 @@
         <f>IF(OR(E56="",L56=""),"",IF(AND(L56&gt;=VLOOKUP(E56,Tiers!$A$4:$C$7,2,0),L56&lt;=VLOOKUP(E56,Tiers!$A$4:$C$7,3,0)),"OK","Fora"))</f>
         <v/>
       </c>
-      <c r="N56" s="5" t="n"/>
-      <c r="O56" s="5" t="n"/>
+      <c r="N56" s="5" t="inlineStr">
+        <is>
+          <t>Campeão</t>
+        </is>
+      </c>
+      <c r="O56" s="5" t="inlineStr">
+        <is>
+          <t>relíquia máxima</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr"/>
+      <c r="B57" s="5" t="inlineStr"/>
+      <c r="C57" s="5" t="inlineStr"/>
+      <c r="D57" s="5" t="inlineStr"/>
+      <c r="E57" s="4" t="inlineStr"/>
+      <c r="F57" s="4" t="inlineStr"/>
+      <c r="G57" s="5" t="inlineStr"/>
+      <c r="H57" s="4" t="inlineStr"/>
+      <c r="I57" s="4" t="inlineStr"/>
+      <c r="J57" s="4" t="inlineStr"/>
+      <c r="K57" s="4" t="inlineStr"/>
+      <c r="L57" s="4">
+        <f>IF(COUNT(H57:K57)=4,SUM(H57:K57),"")</f>
+        <v/>
+      </c>
+      <c r="M57" s="4">
+        <f>IF(OR(E57="",L57=""),"",IF(AND(L57&gt;=VLOOKUP(E57,Tiers!$A$4:$C$7,2,0),L57&lt;=VLOOKUP(E57,Tiers!$A$4:$C$7,3,0)),"OK","Fora"))</f>
+        <v/>
+      </c>
+      <c r="N57" s="5" t="n"/>
+      <c r="O57" s="5" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr"/>
+      <c r="B58" s="5" t="inlineStr"/>
+      <c r="C58" s="5" t="inlineStr"/>
+      <c r="D58" s="5" t="inlineStr"/>
+      <c r="E58" s="4" t="inlineStr"/>
+      <c r="F58" s="4" t="inlineStr"/>
+      <c r="G58" s="5" t="inlineStr"/>
+      <c r="H58" s="4" t="inlineStr"/>
+      <c r="I58" s="4" t="inlineStr"/>
+      <c r="J58" s="4" t="inlineStr"/>
+      <c r="K58" s="4" t="inlineStr"/>
+      <c r="L58" s="4">
+        <f>IF(COUNT(H58:K58)=4,SUM(H58:K58),"")</f>
+        <v/>
+      </c>
+      <c r="M58" s="4">
+        <f>IF(OR(E58="",L58=""),"",IF(AND(L58&gt;=VLOOKUP(E58,Tiers!$A$4:$C$7,2,0),L58&lt;=VLOOKUP(E58,Tiers!$A$4:$C$7,3,0)),"OK","Fora"))</f>
+        <v/>
+      </c>
+      <c r="N58" s="5" t="n"/>
+      <c r="O58" s="5" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr"/>
+      <c r="B59" s="5" t="inlineStr"/>
+      <c r="C59" s="5" t="inlineStr"/>
+      <c r="D59" s="5" t="inlineStr"/>
+      <c r="E59" s="4" t="inlineStr"/>
+      <c r="F59" s="4" t="inlineStr"/>
+      <c r="G59" s="5" t="inlineStr"/>
+      <c r="H59" s="4" t="inlineStr"/>
+      <c r="I59" s="4" t="inlineStr"/>
+      <c r="J59" s="4" t="inlineStr"/>
+      <c r="K59" s="4" t="inlineStr"/>
+      <c r="L59" s="4">
+        <f>IF(COUNT(H59:K59)=4,SUM(H59:K59),"")</f>
+        <v/>
+      </c>
+      <c r="M59" s="4">
+        <f>IF(OR(E59="",L59=""),"",IF(AND(L59&gt;=VLOOKUP(E59,Tiers!$A$4:$C$7,2,0),L59&lt;=VLOOKUP(E59,Tiers!$A$4:$C$7,3,0)),"OK","Fora"))</f>
+        <v/>
+      </c>
+      <c r="N59" s="5" t="n"/>
+      <c r="O59" s="5" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr"/>
+      <c r="B60" s="5" t="inlineStr"/>
+      <c r="C60" s="5" t="inlineStr"/>
+      <c r="D60" s="5" t="inlineStr"/>
+      <c r="E60" s="4" t="inlineStr"/>
+      <c r="F60" s="4" t="inlineStr"/>
+      <c r="G60" s="5" t="inlineStr"/>
+      <c r="H60" s="4" t="inlineStr"/>
+      <c r="I60" s="4" t="inlineStr"/>
+      <c r="J60" s="4" t="inlineStr"/>
+      <c r="K60" s="4" t="inlineStr"/>
+      <c r="L60" s="4">
+        <f>IF(COUNT(H60:K60)=4,SUM(H60:K60),"")</f>
+        <v/>
+      </c>
+      <c r="M60" s="4">
+        <f>IF(OR(E60="",L60=""),"",IF(AND(L60&gt;=VLOOKUP(E60,Tiers!$A$4:$C$7,2,0),L60&lt;=VLOOKUP(E60,Tiers!$A$4:$C$7,3,0)),"OK","Fora"))</f>
+        <v/>
+      </c>
+      <c r="N60" s="5" t="n"/>
+      <c r="O60" s="5" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr"/>
+      <c r="B61" s="5" t="inlineStr"/>
+      <c r="C61" s="5" t="inlineStr"/>
+      <c r="D61" s="5" t="inlineStr"/>
+      <c r="E61" s="4" t="inlineStr"/>
+      <c r="F61" s="4" t="inlineStr"/>
+      <c r="G61" s="5" t="inlineStr"/>
+      <c r="H61" s="4" t="inlineStr"/>
+      <c r="I61" s="4" t="inlineStr"/>
+      <c r="J61" s="4" t="inlineStr"/>
+      <c r="K61" s="4" t="inlineStr"/>
+      <c r="L61" s="4">
+        <f>IF(COUNT(H61:K61)=4,SUM(H61:K61),"")</f>
+        <v/>
+      </c>
+      <c r="M61" s="4">
+        <f>IF(OR(E61="",L61=""),"",IF(AND(L61&gt;=VLOOKUP(E61,Tiers!$A$4:$C$7,2,0),L61&lt;=VLOOKUP(E61,Tiers!$A$4:$C$7,3,0)),"OK","Fora"))</f>
+        <v/>
+      </c>
+      <c r="N61" s="5" t="n"/>
+      <c r="O61" s="5" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr"/>
+      <c r="B62" s="5" t="inlineStr"/>
+      <c r="C62" s="5" t="inlineStr"/>
+      <c r="D62" s="5" t="inlineStr"/>
+      <c r="E62" s="4" t="inlineStr"/>
+      <c r="F62" s="4" t="inlineStr"/>
+      <c r="G62" s="5" t="inlineStr"/>
+      <c r="H62" s="4" t="inlineStr"/>
+      <c r="I62" s="4" t="inlineStr"/>
+      <c r="J62" s="4" t="inlineStr"/>
+      <c r="K62" s="4" t="inlineStr"/>
+      <c r="L62" s="4">
+        <f>IF(COUNT(H62:K62)=4,SUM(H62:K62),"")</f>
+        <v/>
+      </c>
+      <c r="M62" s="4">
+        <f>IF(OR(E62="",L62=""),"",IF(AND(L62&gt;=VLOOKUP(E62,Tiers!$A$4:$C$7,2,0),L62&lt;=VLOOKUP(E62,Tiers!$A$4:$C$7,3,0)),"OK","Fora"))</f>
+        <v/>
+      </c>
+      <c r="N62" s="5" t="n"/>
+      <c r="O62" s="5" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="4">
-    <dataValidation sqref="D5:D56" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Valor inválido" type="list">
+    <dataValidation sqref="D5:D62" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Valor inválido" type="list">
       <formula1>"Crop,Forrageável,Animal,Peixe,Monstro,Mineral,Prato,Aldeão,Especial"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E56" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Valor inválido" type="list">
+    <dataValidation sqref="E5:E62" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Valor inválido" type="list">
       <formula1>"Comum,Incomum,Raro,Lendário"</formula1>
     </dataValidation>
-    <dataValidation sqref="F5:F56" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Valor inválido" type="list">
+    <dataValidation sqref="F5:F62" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Valor inválido" type="list">
       <formula1>"Primavera,Verão,Outono,Inverno,Nenhum"</formula1>
     </dataValidation>
-    <dataValidation sqref="H5:H56 I5:I56 J5:J56 K5:K56" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Bordas devem ser de 1 a 10" type="whole" operator="between">
+    <dataValidation sqref="H5:H62 I5:I62 J5:J62 K5:K62" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Bordas devem ser de 1 a 10" type="whole" operator="between">
       <formula1>1</formula1>
       <formula2>10</formula2>
     </dataValidation>
@@ -2813,14 +4293,14 @@
     <row r="15">
       <c r="A15" s="16" t="inlineStr">
         <is>
-          <t>Convenção de Sprite:</t>
+          <t>Nota:</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>(O)&lt;id&gt; = objeto por Item ID  ·  Villager:&lt;Nome&gt;  ·  Animal:&lt;Tipo&gt;  ·  Monster:&lt;Tipo&gt;  ·  Special:&lt;Nome&gt;</t>
+          <t>IDs de item usam os IDs de objeto legados do SDV (ainda válidos como (O)&lt;id&gt; no 1.6). Estações vêm das páginas Crops/Foraging; conferir antes de fechar o balanceamento.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Valley Triad: balance card stat lines; validate item IDs vs game data
- Verified all 26 object IDs in cards.xlsx against the installed game's
  Content/Data/Objects.xnb (v1.6.15, LZX-decompressed) -- every (O)id matches
  its internal Name.
- Balancing pass on all 52 stat lines: power scales within each tier and each
  card has a distinct edge shape (directional peak + weak opposite). Spread:
  Common 8-14, Uncommon 17-21, Rare 24-28, Legendary 32-36; none out of budget.
- RULES.md: note the validation provenance and balancing approach.
</commit_message>
<xml_diff>
--- a/ValleyTriad/cards.xlsx
+++ b/ValleyTriad/cards.xlsx
@@ -806,10 +806,10 @@
         <v>3</v>
       </c>
       <c r="I5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" s="4" t="n">
         <v>2</v>
-      </c>
-      <c r="J5" s="4" t="n">
-        <v>4</v>
       </c>
       <c r="K5" s="4" t="n">
         <v>2</v>
@@ -829,7 +829,7 @@
       </c>
       <c r="O5" s="5" t="inlineStr">
         <is>
-          <t>starter</t>
+          <t>starter fraco</t>
         </is>
       </c>
     </row>
@@ -868,16 +868,16 @@
         </is>
       </c>
       <c r="H6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I6" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="I6" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="J6" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="K6" s="4" t="n">
         <v>2</v>
-      </c>
-      <c r="K6" s="4" t="n">
-        <v>3</v>
       </c>
       <c r="L6" s="4">
         <f>IF(COUNT(H6:K6)=4,SUM(H6:K6),"")</f>
@@ -892,7 +892,11 @@
           <t>Pacote inicial</t>
         </is>
       </c>
-      <c r="O6" s="5" t="inlineStr"/>
+      <c r="O6" s="5" t="inlineStr">
+        <is>
+          <t>crop grande</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
@@ -935,7 +939,7 @@
         <v>3</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K7" s="4" t="n">
         <v>2</v>
@@ -953,7 +957,11 @@
           <t>Pacote inicial</t>
         </is>
       </c>
-      <c r="O7" s="5" t="inlineStr"/>
+      <c r="O7" s="5" t="inlineStr">
+        <is>
+          <t>arredondada</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
@@ -993,10 +1001,10 @@
         <v>2</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K8" s="4" t="n">
         <v>2</v>
@@ -1014,7 +1022,11 @@
           <t>Ganhar de NPC</t>
         </is>
       </c>
-      <c r="O8" s="5" t="inlineStr"/>
+      <c r="O8" s="5" t="inlineStr">
+        <is>
+          <t>pico à direita</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
@@ -1051,16 +1063,16 @@
         </is>
       </c>
       <c r="H9" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="I9" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="I9" s="4" t="n">
+      <c r="J9" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="J9" s="4" t="n">
+      <c r="K9" s="4" t="n">
         <v>3</v>
-      </c>
-      <c r="K9" s="4" t="n">
-        <v>4</v>
       </c>
       <c r="L9" s="4">
         <f>IF(COUNT(H9:K9)=4,SUM(H9:K9),"")</f>
@@ -1075,7 +1087,11 @@
           <t>Pacote inicial</t>
         </is>
       </c>
-      <c r="O9" s="5" t="inlineStr"/>
+      <c r="O9" s="5" t="inlineStr">
+        <is>
+          <t>vertical</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
@@ -1118,10 +1134,10 @@
         <v>2</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L10" s="4">
         <f>IF(COUNT(H10:K10)=4,SUM(H10:K10),"")</f>
@@ -1136,7 +1152,11 @@
           <t>Ganhar de NPC</t>
         </is>
       </c>
-      <c r="O10" s="5" t="inlineStr"/>
+      <c r="O10" s="5" t="inlineStr">
+        <is>
+          <t>pico no topo</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
@@ -1179,10 +1199,10 @@
         <v>4</v>
       </c>
       <c r="J11" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K11" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L11" s="4">
         <f>IF(COUNT(H11:K11)=4,SUM(H11:K11),"")</f>
@@ -1197,7 +1217,11 @@
           <t>Ganhar de NPC</t>
         </is>
       </c>
-      <c r="O11" s="5" t="inlineStr"/>
+      <c r="O11" s="5" t="inlineStr">
+        <is>
+          <t>fruta grande</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
@@ -1304,7 +1328,7 @@
         <v>4</v>
       </c>
       <c r="K13" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L13" s="4">
         <f>IF(COUNT(H13:K13)=4,SUM(H13:K13),"")</f>
@@ -1321,7 +1345,7 @@
       </c>
       <c r="O13" s="5" t="inlineStr">
         <is>
-          <t>forte em casa de Outono</t>
+          <t>topo forte; casa de Outono</t>
         </is>
       </c>
     </row>
@@ -1366,10 +1390,10 @@
         <v>4</v>
       </c>
       <c r="J14" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="K14" s="4" t="n">
         <v>4</v>
-      </c>
-      <c r="K14" s="4" t="n">
-        <v>3</v>
       </c>
       <c r="L14" s="4">
         <f>IF(COUNT(H14:K14)=4,SUM(H14:K14),"")</f>
@@ -1384,7 +1408,11 @@
           <t>Ganhar de NPC</t>
         </is>
       </c>
-      <c r="O14" s="5" t="inlineStr"/>
+      <c r="O14" s="5" t="inlineStr">
+        <is>
+          <t>horizontal</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
@@ -1427,7 +1455,7 @@
         <v>3</v>
       </c>
       <c r="J15" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K15" s="4" t="n">
         <v>2</v>
@@ -1488,10 +1516,10 @@
         <v>2</v>
       </c>
       <c r="J16" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K16" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L16" s="4">
         <f>IF(COUNT(H16:K16)=4,SUM(H16:K16),"")</f>
@@ -1506,7 +1534,11 @@
           <t>Pacote inicial</t>
         </is>
       </c>
-      <c r="O16" s="5" t="inlineStr"/>
+      <c r="O16" s="5" t="inlineStr">
+        <is>
+          <t>raiz: pico embaixo</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
@@ -1552,7 +1584,7 @@
         <v>2</v>
       </c>
       <c r="K17" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L17" s="4">
         <f>IF(COUNT(H17:K17)=4,SUM(H17:K17),"")</f>
@@ -1613,7 +1645,7 @@
         <v>3</v>
       </c>
       <c r="K18" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L18" s="4">
         <f>IF(COUNT(H18:K18)=4,SUM(H18:K18),"")</f>
@@ -1671,7 +1703,7 @@
         <v>2</v>
       </c>
       <c r="J19" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K19" s="4" t="n">
         <v>2</v>
@@ -1735,7 +1767,7 @@
         <v>2</v>
       </c>
       <c r="K20" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L20" s="4">
         <f>IF(COUNT(H20:K20)=4,SUM(H20:K20),"")</f>
@@ -1854,7 +1886,7 @@
         <v>2</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K22" s="4" t="n">
         <v>2</v>
@@ -1872,7 +1904,11 @@
           <t>Ganhar de NPC</t>
         </is>
       </c>
-      <c r="O22" s="5" t="inlineStr"/>
+      <c r="O22" s="5" t="inlineStr">
+        <is>
+          <t>raro no Inverno</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
@@ -1915,10 +1951,10 @@
         <v>3</v>
       </c>
       <c r="J23" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K23" s="4" t="n">
         <v>3</v>
-      </c>
-      <c r="K23" s="4" t="n">
-        <v>2</v>
       </c>
       <c r="L23" s="4">
         <f>IF(COUNT(H23:K23)=4,SUM(H23:K23),"")</f>
@@ -1976,10 +2012,10 @@
         <v>2</v>
       </c>
       <c r="J24" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K24" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L24" s="4">
         <f>IF(COUNT(H24:K24)=4,SUM(H24:K24),"")</f>
@@ -2037,10 +2073,10 @@
         <v>3</v>
       </c>
       <c r="J25" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="K25" s="4" t="n">
         <v>3</v>
-      </c>
-      <c r="K25" s="4" t="n">
-        <v>4</v>
       </c>
       <c r="L25" s="4">
         <f>IF(COUNT(H25:K25)=4,SUM(H25:K25),"")</f>
@@ -2055,7 +2091,11 @@
           <t>Ganhar de NPC</t>
         </is>
       </c>
-      <c r="O25" s="5" t="inlineStr"/>
+      <c r="O25" s="5" t="inlineStr">
+        <is>
+          <t>animal grande</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
@@ -2095,10 +2135,10 @@
         <v>3</v>
       </c>
       <c r="I26" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J26" s="4" t="n">
         <v>2</v>
-      </c>
-      <c r="J26" s="4" t="n">
-        <v>3</v>
       </c>
       <c r="K26" s="4" t="n">
         <v>3</v>
@@ -2159,10 +2199,10 @@
         <v>4</v>
       </c>
       <c r="J27" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K27" s="4" t="n">
         <v>3</v>
-      </c>
-      <c r="K27" s="4" t="n">
-        <v>2</v>
       </c>
       <c r="L27" s="4">
         <f>IF(COUNT(H27:K27)=4,SUM(H27:K27),"")</f>
@@ -2177,7 +2217,11 @@
           <t>Ganhar de NPC</t>
         </is>
       </c>
-      <c r="O27" s="5" t="inlineStr"/>
+      <c r="O27" s="5" t="inlineStr">
+        <is>
+          <t>ágil: laterais</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
@@ -2214,10 +2258,10 @@
         </is>
       </c>
       <c r="H28" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I28" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J28" s="4" t="n">
         <v>2</v>
@@ -2238,7 +2282,11 @@
           <t>Ganhar de NPC</t>
         </is>
       </c>
-      <c r="O28" s="5" t="inlineStr"/>
+      <c r="O28" s="5" t="inlineStr">
+        <is>
+          <t>cristal: horizontal</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
@@ -2278,7 +2326,7 @@
         <v>6</v>
       </c>
       <c r="I29" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J29" s="4" t="n">
         <v>4</v>
@@ -2349,7 +2397,7 @@
         <v>5</v>
       </c>
       <c r="K30" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L30" s="4">
         <f>IF(COUNT(H30:K30)=4,SUM(H30:K30),"")</f>
@@ -2404,10 +2452,10 @@
         <v>5</v>
       </c>
       <c r="I31" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J31" s="4" t="n">
         <v>4</v>
-      </c>
-      <c r="J31" s="4" t="n">
-        <v>5</v>
       </c>
       <c r="K31" s="4" t="n">
         <v>4</v>
@@ -2465,10 +2513,10 @@
         <v>4</v>
       </c>
       <c r="I32" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J32" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K32" s="4" t="n">
         <v>4</v>
@@ -2486,7 +2534,11 @@
           <t>Ganhar de NPC</t>
         </is>
       </c>
-      <c r="O32" s="5" t="inlineStr"/>
+      <c r="O32" s="5" t="inlineStr">
+        <is>
+          <t>acolhedora: base forte</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
@@ -2529,10 +2581,10 @@
         <v>4</v>
       </c>
       <c r="J33" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="K33" s="4" t="n">
         <v>4</v>
-      </c>
-      <c r="K33" s="4" t="n">
-        <v>5</v>
       </c>
       <c r="L33" s="4">
         <f>IF(COUNT(H33:K33)=4,SUM(H33:K33),"")</f>
@@ -2608,7 +2660,11 @@
           <t>Ganhar de NPC</t>
         </is>
       </c>
-      <c r="O34" s="5" t="inlineStr"/>
+      <c r="O34" s="5" t="inlineStr">
+        <is>
+          <t>eloquente: direita</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
@@ -2645,13 +2701,13 @@
         </is>
       </c>
       <c r="H35" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I35" s="4" t="n">
         <v>4</v>
       </c>
       <c r="J35" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K35" s="4" t="n">
         <v>4</v>
@@ -2712,7 +2768,7 @@
         <v>5</v>
       </c>
       <c r="J36" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K36" s="4" t="n">
         <v>5</v>
@@ -2730,7 +2786,11 @@
           <t>Ganhar de NPC</t>
         </is>
       </c>
-      <c r="O36" s="5" t="inlineStr"/>
+      <c r="O36" s="5" t="inlineStr">
+        <is>
+          <t>engenheira: equilibrada</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="n">
@@ -2852,7 +2912,11 @@
           <t>Ganhar de NPC</t>
         </is>
       </c>
-      <c r="O38" s="5" t="inlineStr"/>
+      <c r="O38" s="5" t="inlineStr">
+        <is>
+          <t>pico no topo</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="n">
@@ -2889,7 +2953,7 @@
         </is>
       </c>
       <c r="H39" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I39" s="4" t="n">
         <v>5</v>
@@ -2915,7 +2979,7 @@
       </c>
       <c r="O39" s="5" t="inlineStr">
         <is>
-          <t>dono do Saloon</t>
+          <t>dono do Saloon; robusto</t>
         </is>
       </c>
     </row>
@@ -2978,7 +3042,11 @@
           <t>Ganhar de NPC</t>
         </is>
       </c>
-      <c r="O40" s="5" t="inlineStr"/>
+      <c r="O40" s="5" t="inlineStr">
+        <is>
+          <t>mediano</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="n">
@@ -3015,7 +3083,7 @@
         </is>
       </c>
       <c r="H41" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I41" s="4" t="n">
         <v>5</v>
@@ -3039,7 +3107,11 @@
           <t>Ganhar de NPC</t>
         </is>
       </c>
-      <c r="O41" s="5" t="inlineStr"/>
+      <c r="O41" s="5" t="inlineStr">
+        <is>
+          <t>carpinteira: sólida</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="n">
@@ -3079,13 +3151,13 @@
         <v>6</v>
       </c>
       <c r="I42" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J42" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="J42" s="4" t="n">
+      <c r="K42" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="K42" s="4" t="n">
-        <v>4</v>
       </c>
       <c r="L42" s="4">
         <f>IF(COUNT(H42:K42)=4,SUM(H42:K42),"")</f>
@@ -3100,7 +3172,11 @@
           <t>Ganhar de NPC</t>
         </is>
       </c>
-      <c r="O42" s="5" t="inlineStr"/>
+      <c r="O42" s="5" t="inlineStr">
+        <is>
+          <t>ferreiro: forte</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="n">
@@ -3146,7 +3222,7 @@
         <v>4</v>
       </c>
       <c r="K43" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L43" s="4">
         <f>IF(COUNT(H43:K43)=4,SUM(H43:K43),"")</f>
@@ -3161,7 +3237,11 @@
           <t>Ganhar de NPC</t>
         </is>
       </c>
-      <c r="O43" s="5" t="inlineStr"/>
+      <c r="O43" s="5" t="inlineStr">
+        <is>
+          <t>pescador</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="n">
@@ -3204,10 +3284,10 @@
         <v>6</v>
       </c>
       <c r="J44" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="K44" s="4" t="n">
         <v>5</v>
-      </c>
-      <c r="K44" s="4" t="n">
-        <v>6</v>
       </c>
       <c r="L44" s="4">
         <f>IF(COUNT(H44:K44)=4,SUM(H44:K44),"")</f>
@@ -3283,7 +3363,11 @@
           <t>Ganhar de NPC</t>
         </is>
       </c>
-      <c r="O45" s="5" t="inlineStr"/>
+      <c r="O45" s="5" t="inlineStr">
+        <is>
+          <t>agressivo: topo</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="n">
@@ -3323,13 +3407,13 @@
         <v>6</v>
       </c>
       <c r="I46" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J46" s="4" t="n">
         <v>6</v>
       </c>
       <c r="K46" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L46" s="4">
         <f>IF(COUNT(H46:K46)=4,SUM(H46:K46),"")</f>
@@ -3344,7 +3428,11 @@
           <t>Ganhar de NPC</t>
         </is>
       </c>
-      <c r="O46" s="5" t="inlineStr"/>
+      <c r="O46" s="5" t="inlineStr">
+        <is>
+          <t>veloz: direita</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="n">
@@ -3387,10 +3475,10 @@
         <v>7</v>
       </c>
       <c r="J47" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K47" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L47" s="4">
         <f>IF(COUNT(H47:K47)=4,SUM(H47:K47),"")</f>
@@ -3407,7 +3495,7 @@
       </c>
       <c r="O47" s="5" t="inlineStr">
         <is>
-          <t>dino das cavernas</t>
+          <t>dino poderoso</t>
         </is>
       </c>
     </row>
@@ -3470,7 +3558,11 @@
           <t>Ganhar de NPC</t>
         </is>
       </c>
-      <c r="O48" s="5" t="inlineStr"/>
+      <c r="O48" s="5" t="inlineStr">
+        <is>
+          <t>equilíbrio alto</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="n">
@@ -3574,7 +3666,7 @@
         <v>6</v>
       </c>
       <c r="J50" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K50" s="4" t="n">
         <v>5</v>
@@ -3592,7 +3684,11 @@
           <t>Ganhar de NPC</t>
         </is>
       </c>
-      <c r="O50" s="5" t="inlineStr"/>
+      <c r="O50" s="5" t="inlineStr">
+        <is>
+          <t>peixe grande: base</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="n">
@@ -3632,7 +3728,7 @@
         <v>8</v>
       </c>
       <c r="I51" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J51" s="4" t="n">
         <v>7</v>
@@ -3653,7 +3749,11 @@
           <t>Ganhar de NPC</t>
         </is>
       </c>
-      <c r="O51" s="5" t="inlineStr"/>
+      <c r="O51" s="5" t="inlineStr">
+        <is>
+          <t>premium do tier</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="n">
@@ -3823,7 +3923,7 @@
         <v>10</v>
       </c>
       <c r="I54" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J54" s="4" t="n">
         <v>8</v>
@@ -3846,7 +3946,7 @@
       </c>
       <c r="O54" s="5" t="inlineStr">
         <is>
-          <t>boss</t>
+          <t>boss supremo</t>
         </is>
       </c>
     </row>
@@ -3894,7 +3994,7 @@
         <v>9</v>
       </c>
       <c r="K55" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L55" s="4">
         <f>IF(COUNT(H55:K55)=4,SUM(H55:K55),"")</f>
@@ -3956,10 +4056,10 @@
         <v>9</v>
       </c>
       <c r="J56" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="K56" s="4" t="n">
         <v>8</v>
-      </c>
-      <c r="K56" s="4" t="n">
-        <v>9</v>
       </c>
       <c r="L56" s="4">
         <f>IF(COUNT(H56:K56)=4,SUM(H56:K56),"")</f>
@@ -4300,7 +4400,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>IDs de item usam os IDs de objeto legados do SDV (ainda válidos como (O)&lt;id&gt; no 1.6). Estações vêm das páginas Crops/Foraging; conferir antes de fechar o balanceamento.</t>
+          <t>IDs de objeto VALIDADOS contra o Content/Data/Objects.xnb do jogo instalado (v1.6.15) — cada (O)&lt;id&gt; confere com o Name interno. Estações das páginas Crops/Foraging.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Valley Triad: add game-sourced SpriteIndex/price columns + generator tools
- cards.xlsx: new SpriteIndex and Price columns for object cards, extracted from
  the installed game's Content/Data/Objects.xnb (v1.6.15). Villager/animal/monster
  cards leave them blank (sourced from other data files).
- tools/: reproducible generators (build_cards.py for the sheet, render_cards.py for
  preview cards). No game assets committed.
- .gitignore: exclude card-previews/ (composed from © ConcernedApe sprites; kept
  local only — the mod composes sprites at runtime from the player's own files).
</commit_message>
<xml_diff>
--- a/ValleyTriad/cards.xlsx
+++ b/ValleyTriad/cards.xlsx
@@ -657,7 +657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O62"/>
+  <dimension ref="A1:Q62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -675,6 +675,8 @@
     <col width="11" customWidth="1" min="13" max="13"/>
     <col width="15" customWidth="1" min="14" max="14"/>
     <col width="26" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -767,6 +769,16 @@
           <t>Notas</t>
         </is>
       </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>SpriteIndex</t>
+        </is>
+      </c>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>Preço (g)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
@@ -832,6 +844,12 @@
           <t>starter fraco</t>
         </is>
       </c>
+      <c r="P5" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="Q5" s="4" t="n">
+        <v>35</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
@@ -897,6 +915,12 @@
           <t>crop grande</t>
         </is>
       </c>
+      <c r="P6" s="4" t="n">
+        <v>190</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>175</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
@@ -962,6 +986,12 @@
           <t>arredondada</t>
         </is>
       </c>
+      <c r="P7" s="4" t="n">
+        <v>192</v>
+      </c>
+      <c r="Q7" s="4" t="n">
+        <v>80</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
@@ -1027,6 +1057,12 @@
           <t>pico à direita</t>
         </is>
       </c>
+      <c r="P8" s="4" t="n">
+        <v>188</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
@@ -1092,6 +1128,12 @@
           <t>vertical</t>
         </is>
       </c>
+      <c r="P9" s="4" t="n">
+        <v>258</v>
+      </c>
+      <c r="Q9" s="4" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
@@ -1157,6 +1199,12 @@
           <t>pico no topo</t>
         </is>
       </c>
+      <c r="P10" s="4" t="n">
+        <v>260</v>
+      </c>
+      <c r="Q10" s="4" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
@@ -1222,6 +1270,12 @@
           <t>fruta grande</t>
         </is>
       </c>
+      <c r="P11" s="4" t="n">
+        <v>254</v>
+      </c>
+      <c r="Q11" s="4" t="n">
+        <v>250</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
@@ -1283,6 +1337,12 @@
         </is>
       </c>
       <c r="O12" s="5" t="inlineStr"/>
+      <c r="P12" s="4" t="n">
+        <v>256</v>
+      </c>
+      <c r="Q12" s="4" t="n">
+        <v>60</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
@@ -1348,6 +1408,12 @@
           <t>topo forte; casa de Outono</t>
         </is>
       </c>
+      <c r="P13" s="4" t="n">
+        <v>276</v>
+      </c>
+      <c r="Q13" s="4" t="n">
+        <v>320</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
@@ -1413,6 +1479,12 @@
           <t>horizontal</t>
         </is>
       </c>
+      <c r="P14" s="4" t="n">
+        <v>282</v>
+      </c>
+      <c r="Q14" s="4" t="n">
+        <v>75</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
@@ -1474,6 +1546,12 @@
         </is>
       </c>
       <c r="O15" s="5" t="inlineStr"/>
+      <c r="P15" s="4" t="n">
+        <v>272</v>
+      </c>
+      <c r="Q15" s="4" t="n">
+        <v>60</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
@@ -1539,6 +1617,12 @@
           <t>raiz: pico embaixo</t>
         </is>
       </c>
+      <c r="P16" s="4" t="n">
+        <v>280</v>
+      </c>
+      <c r="Q16" s="4" t="n">
+        <v>160</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
@@ -1600,6 +1684,12 @@
         </is>
       </c>
       <c r="O17" s="5" t="inlineStr"/>
+      <c r="P17" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="Q17" s="4" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
@@ -1661,6 +1751,12 @@
         </is>
       </c>
       <c r="O18" s="5" t="inlineStr"/>
+      <c r="P18" s="4" t="n">
+        <v>296</v>
+      </c>
+      <c r="Q18" s="4" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
@@ -1722,6 +1818,12 @@
         </is>
       </c>
       <c r="O19" s="5" t="inlineStr"/>
+      <c r="P19" s="4" t="n">
+        <v>396</v>
+      </c>
+      <c r="Q19" s="4" t="n">
+        <v>80</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
@@ -1783,6 +1885,12 @@
         </is>
       </c>
       <c r="O20" s="5" t="inlineStr"/>
+      <c r="P20" s="4" t="n">
+        <v>404</v>
+      </c>
+      <c r="Q20" s="4" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
@@ -1844,6 +1952,12 @@
         </is>
       </c>
       <c r="O21" s="5" t="inlineStr"/>
+      <c r="P21" s="4" t="n">
+        <v>410</v>
+      </c>
+      <c r="Q21" s="4" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
@@ -1909,6 +2023,12 @@
           <t>raro no Inverno</t>
         </is>
       </c>
+      <c r="P22" s="4" t="n">
+        <v>412</v>
+      </c>
+      <c r="Q22" s="4" t="n">
+        <v>70</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
@@ -1970,6 +2090,12 @@
         </is>
       </c>
       <c r="O23" s="5" t="inlineStr"/>
+      <c r="P23" s="4" t="n">
+        <v>416</v>
+      </c>
+      <c r="Q23" s="4" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
@@ -2031,6 +2157,8 @@
         </is>
       </c>
       <c r="O24" s="5" t="inlineStr"/>
+      <c r="P24" s="4" t="n"/>
+      <c r="Q24" s="4" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
@@ -2096,6 +2224,8 @@
           <t>animal grande</t>
         </is>
       </c>
+      <c r="P25" s="4" t="n"/>
+      <c r="Q25" s="4" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
@@ -2157,6 +2287,8 @@
         </is>
       </c>
       <c r="O26" s="5" t="inlineStr"/>
+      <c r="P26" s="4" t="n"/>
+      <c r="Q26" s="4" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
@@ -2222,6 +2354,8 @@
           <t>ágil: laterais</t>
         </is>
       </c>
+      <c r="P27" s="4" t="n"/>
+      <c r="Q27" s="4" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
@@ -2287,6 +2421,12 @@
           <t>cristal: horizontal</t>
         </is>
       </c>
+      <c r="P28" s="4" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q28" s="4" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
@@ -2352,6 +2492,8 @@
           <t>mentora / evento inicial</t>
         </is>
       </c>
+      <c r="P29" s="4" t="n"/>
+      <c r="Q29" s="4" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
@@ -2413,6 +2555,8 @@
         </is>
       </c>
       <c r="O30" s="5" t="inlineStr"/>
+      <c r="P30" s="4" t="n"/>
+      <c r="Q30" s="4" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
@@ -2474,6 +2618,8 @@
         </is>
       </c>
       <c r="O31" s="5" t="inlineStr"/>
+      <c r="P31" s="4" t="n"/>
+      <c r="Q31" s="4" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
@@ -2539,6 +2685,8 @@
           <t>acolhedora: base forte</t>
         </is>
       </c>
+      <c r="P32" s="4" t="n"/>
+      <c r="Q32" s="4" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
@@ -2600,6 +2748,8 @@
         </is>
       </c>
       <c r="O33" s="5" t="inlineStr"/>
+      <c r="P33" s="4" t="n"/>
+      <c r="Q33" s="4" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
@@ -2665,6 +2815,8 @@
           <t>eloquente: direita</t>
         </is>
       </c>
+      <c r="P34" s="4" t="n"/>
+      <c r="Q34" s="4" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
@@ -2726,6 +2878,8 @@
         </is>
       </c>
       <c r="O35" s="5" t="inlineStr"/>
+      <c r="P35" s="4" t="n"/>
+      <c r="Q35" s="4" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="n">
@@ -2791,6 +2945,8 @@
           <t>engenheira: equilibrada</t>
         </is>
       </c>
+      <c r="P36" s="4" t="n"/>
+      <c r="Q36" s="4" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="n">
@@ -2852,6 +3008,8 @@
         </is>
       </c>
       <c r="O37" s="5" t="inlineStr"/>
+      <c r="P37" s="4" t="n"/>
+      <c r="Q37" s="4" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="n">
@@ -2917,6 +3075,8 @@
           <t>pico no topo</t>
         </is>
       </c>
+      <c r="P38" s="4" t="n"/>
+      <c r="Q38" s="4" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="n">
@@ -2982,6 +3142,8 @@
           <t>dono do Saloon; robusto</t>
         </is>
       </c>
+      <c r="P39" s="4" t="n"/>
+      <c r="Q39" s="4" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="n">
@@ -3047,6 +3209,8 @@
           <t>mediano</t>
         </is>
       </c>
+      <c r="P40" s="4" t="n"/>
+      <c r="Q40" s="4" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="n">
@@ -3112,6 +3276,8 @@
           <t>carpinteira: sólida</t>
         </is>
       </c>
+      <c r="P41" s="4" t="n"/>
+      <c r="Q41" s="4" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="4" t="n">
@@ -3177,6 +3343,8 @@
           <t>ferreiro: forte</t>
         </is>
       </c>
+      <c r="P42" s="4" t="n"/>
+      <c r="Q42" s="4" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="n">
@@ -3242,6 +3410,8 @@
           <t>pescador</t>
         </is>
       </c>
+      <c r="P43" s="4" t="n"/>
+      <c r="Q43" s="4" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="4" t="n">
@@ -3303,6 +3473,8 @@
         </is>
       </c>
       <c r="O44" s="5" t="inlineStr"/>
+      <c r="P44" s="4" t="n"/>
+      <c r="Q44" s="4" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="n">
@@ -3368,6 +3540,8 @@
           <t>agressivo: topo</t>
         </is>
       </c>
+      <c r="P45" s="4" t="n"/>
+      <c r="Q45" s="4" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="4" t="n">
@@ -3433,6 +3607,8 @@
           <t>veloz: direita</t>
         </is>
       </c>
+      <c r="P46" s="4" t="n"/>
+      <c r="Q46" s="4" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="n">
@@ -3498,6 +3674,8 @@
           <t>dino poderoso</t>
         </is>
       </c>
+      <c r="P47" s="4" t="n"/>
+      <c r="Q47" s="4" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="4" t="n">
@@ -3563,6 +3741,12 @@
           <t>equilíbrio alto</t>
         </is>
       </c>
+      <c r="P48" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="Q48" s="4" t="n">
+        <v>750</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="n">
@@ -3624,6 +3808,12 @@
         </is>
       </c>
       <c r="O49" s="5" t="inlineStr"/>
+      <c r="P49" s="4" t="n">
+        <v>454</v>
+      </c>
+      <c r="Q49" s="4" t="n">
+        <v>550</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="n">
@@ -3689,6 +3879,12 @@
           <t>peixe grande: base</t>
         </is>
       </c>
+      <c r="P50" s="4" t="n">
+        <v>698</v>
+      </c>
+      <c r="Q50" s="4" t="n">
+        <v>200</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="n">
@@ -3754,6 +3950,12 @@
           <t>premium do tier</t>
         </is>
       </c>
+      <c r="P51" s="4" t="n">
+        <v>417</v>
+      </c>
+      <c r="Q51" s="4" t="n">
+        <v>3000</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="n">
@@ -3819,6 +4021,8 @@
           <t>boss</t>
         </is>
       </c>
+      <c r="P52" s="4" t="n"/>
+      <c r="Q52" s="4" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="4" t="n">
@@ -3884,6 +4088,8 @@
           <t>boss</t>
         </is>
       </c>
+      <c r="P53" s="4" t="n"/>
+      <c r="Q53" s="4" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="4" t="n">
@@ -3949,6 +4155,8 @@
           <t>boss supremo</t>
         </is>
       </c>
+      <c r="P54" s="4" t="n"/>
+      <c r="Q54" s="4" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="4" t="n">
@@ -4014,6 +4222,12 @@
           <t>peixe lendário</t>
         </is>
       </c>
+      <c r="P55" s="4" t="n">
+        <v>159</v>
+      </c>
+      <c r="Q55" s="4" t="n">
+        <v>1500</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="n">
@@ -4078,6 +4292,12 @@
         <is>
           <t>relíquia máxima</t>
         </is>
+      </c>
+      <c r="P56" s="4" t="n">
+        <v>74</v>
+      </c>
+      <c r="Q56" s="4" t="n">
+        <v>2000</v>
       </c>
     </row>
     <row r="57">
@@ -4102,6 +4322,8 @@
       </c>
       <c r="N57" s="5" t="n"/>
       <c r="O57" s="5" t="n"/>
+      <c r="P57" s="4" t="n"/>
+      <c r="Q57" s="4" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr"/>
@@ -4125,6 +4347,8 @@
       </c>
       <c r="N58" s="5" t="n"/>
       <c r="O58" s="5" t="n"/>
+      <c r="P58" s="4" t="n"/>
+      <c r="Q58" s="4" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr"/>
@@ -4148,6 +4372,8 @@
       </c>
       <c r="N59" s="5" t="n"/>
       <c r="O59" s="5" t="n"/>
+      <c r="P59" s="4" t="n"/>
+      <c r="Q59" s="4" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr"/>
@@ -4171,6 +4397,8 @@
       </c>
       <c r="N60" s="5" t="n"/>
       <c r="O60" s="5" t="n"/>
+      <c r="P60" s="4" t="n"/>
+      <c r="Q60" s="4" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr"/>
@@ -4194,6 +4422,8 @@
       </c>
       <c r="N61" s="5" t="n"/>
       <c r="O61" s="5" t="n"/>
+      <c r="P61" s="4" t="n"/>
+      <c r="Q61" s="4" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr"/>
@@ -4217,6 +4447,8 @@
       </c>
       <c r="N62" s="5" t="n"/>
       <c r="O62" s="5" t="n"/>
+      <c r="P62" s="4" t="n"/>
+      <c r="Q62" s="4" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="4">

</xml_diff>